<commit_message>
Site guncellemesi - 09.09.2026 19:36
</commit_message>
<xml_diff>
--- a/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
+++ b/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
@@ -176,6 +176,9 @@
   </x:si>
   <x:si>
     <x:t>14.07.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09.09.2026</x:t>
   </x:si>
   <x:si>
     <x:t>ARSAN</x:t>
@@ -1418,7 +1421,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>8.6</x:v>
+        <x:v>8.94</x:v>
       </x:c>
       <x:c r="J2" s="0">
         <x:v>0</x:v>
@@ -1450,7 +1453,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>4.6</x:v>
+        <x:v>4.72</x:v>
       </x:c>
       <x:c r="J3" s="0">
         <x:v>0</x:v>
@@ -1482,7 +1485,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>6.91</x:v>
+        <x:v>6.65</x:v>
       </x:c>
       <x:c r="J4" s="0">
         <x:v>0</x:v>
@@ -1514,7 +1517,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>9.15</x:v>
+        <x:v>9.23</x:v>
       </x:c>
       <x:c r="J5" s="0">
         <x:v>8.74</x:v>
@@ -1549,7 +1552,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>26.9</x:v>
+        <x:v>27.46</x:v>
       </x:c>
       <x:c r="J6" s="0">
         <x:v>0</x:v>
@@ -1581,7 +1584,7 @@
         <x:v>3.7</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>6.8</x:v>
+        <x:v>6.63</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>6.99</x:v>
@@ -1616,7 +1619,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>21.34</x:v>
+        <x:v>21.18</x:v>
       </x:c>
       <x:c r="J8" s="0">
         <x:v>23.68</x:v>
@@ -1651,7 +1654,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>7.06</x:v>
+        <x:v>7.24</x:v>
       </x:c>
       <x:c r="J9" s="0">
         <x:v>8.39</x:v>
@@ -1686,7 +1689,7 @@
         <x:v>3.83</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>13.65</x:v>
+        <x:v>13.74</x:v>
       </x:c>
       <x:c r="J10" s="0">
         <x:v>0.76</x:v>
@@ -1756,7 +1759,7 @@
         <x:v>8.08</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>15.69</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J12" s="0">
         <x:v>0.73</x:v>
@@ -1791,7 +1794,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>67.3</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="J13" s="0">
         <x:v>64.98</x:v>
@@ -1861,7 +1864,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>138.5</x:v>
+        <x:v>136.4</x:v>
       </x:c>
       <x:c r="J15" s="0">
         <x:v>0</x:v>
@@ -1893,7 +1896,7 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>5.59</x:v>
+        <x:v>5.54</x:v>
       </x:c>
       <x:c r="J16" s="0">
         <x:v>6.13</x:v>
@@ -1928,7 +1931,7 @@
         <x:v>0.43</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>9.87</x:v>
+        <x:v>10.01</x:v>
       </x:c>
       <x:c r="J17" s="0">
         <x:v>9.9</x:v>
@@ -1963,7 +1966,7 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>9.15</x:v>
+        <x:v>9.23</x:v>
       </x:c>
       <x:c r="J18" s="0">
         <x:v>9.69</x:v>
@@ -1998,7 +2001,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>18.6</x:v>
+        <x:v>18.8</x:v>
       </x:c>
       <x:c r="J19" s="0">
         <x:v>0</x:v>
@@ -2030,7 +2033,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>1.68</x:v>
+        <x:v>1.7</x:v>
       </x:c>
       <x:c r="J20" s="0">
         <x:v>0</x:v>
@@ -2062,7 +2065,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>18.13</x:v>
+        <x:v>16.52</x:v>
       </x:c>
       <x:c r="J21" s="0">
         <x:v>15.87</x:v>
@@ -2079,7 +2082,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="C22" s="0">
-        <x:v>4350000</x:v>
+        <x:v>4540000</x:v>
       </x:c>
       <x:c r="D22" s="0">
         <x:v>40000000</x:v>
@@ -2088,30 +2091,30 @@
         <x:v>1000000000</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>83238200</x:v>
+        <x:v>86614200</x:v>
       </x:c>
       <x:c r="G22" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>0.52</x:v>
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>17.98</x:v>
+        <x:v>17.61</x:v>
       </x:c>
       <x:c r="J22" s="0">
-        <x:v>19.14</x:v>
+        <x:v>19.08</x:v>
       </x:c>
       <x:c r="K22" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:11">
       <x:c r="A23" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C23" s="0">
         <x:v>11393782</x:v>
@@ -2132,7 +2135,7 @@
         <x:v>0.65</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>3.92</x:v>
+        <x:v>3.86</x:v>
       </x:c>
       <x:c r="J23" s="0">
         <x:v>3.49</x:v>
@@ -2143,10 +2146,10 @@
     </x:row>
     <x:row r="24" spans="1:11">
       <x:c r="A24" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C24" s="0">
         <x:v>2500000</x:v>
@@ -2167,7 +2170,7 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>420.5</x:v>
+        <x:v>427.5</x:v>
       </x:c>
       <x:c r="J24" s="0">
         <x:v>380.17</x:v>
@@ -2178,10 +2181,10 @@
     </x:row>
     <x:row r="25" spans="1:11">
       <x:c r="A25" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B25" s="0" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="B25" s="0" t="s">
-        <x:v>57</x:v>
       </x:c>
       <x:c r="C25" s="0">
         <x:v>178529</x:v>
@@ -2202,7 +2205,7 @@
         <x:v>1.29</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>77.15</x:v>
+        <x:v>69.5</x:v>
       </x:c>
       <x:c r="J25" s="0">
         <x:v>69.8</x:v>
@@ -2213,10 +2216,10 @@
     </x:row>
     <x:row r="26" spans="1:11">
       <x:c r="A26" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C26" s="0">
         <x:v>2501710</x:v>
@@ -2237,7 +2240,7 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>39.22</x:v>
+        <x:v>39.6</x:v>
       </x:c>
       <x:c r="J26" s="0">
         <x:v>38.82</x:v>
@@ -2248,10 +2251,10 @@
     </x:row>
     <x:row r="27" spans="1:11">
       <x:c r="A27" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C27" s="0">
         <x:v>57675584</x:v>
@@ -2272,21 +2275,21 @@
         <x:v>1.8</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>53</x:v>
+        <x:v>53.9</x:v>
       </x:c>
       <x:c r="J27" s="0">
         <x:v>48.23</x:v>
       </x:c>
       <x:c r="K27" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:11">
       <x:c r="A28" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C28" s="0">
         <x:v>45660619</x:v>
@@ -2307,21 +2310,21 @@
         <x:v>1.55</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>34.9</x:v>
+        <x:v>37.2</x:v>
       </x:c>
       <x:c r="J28" s="0">
         <x:v>34.02</x:v>
       </x:c>
       <x:c r="K28" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:11">
       <x:c r="A29" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C29" s="0">
         <x:v>324474</x:v>
@@ -2342,21 +2345,21 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>15.94</x:v>
+        <x:v>16.43</x:v>
       </x:c>
       <x:c r="J29" s="0">
         <x:v>5.49</x:v>
       </x:c>
       <x:c r="K29" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:11">
       <x:c r="A30" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C30" s="0">
         <x:v>7999148</x:v>
@@ -2377,21 +2380,21 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>24.18</x:v>
+        <x:v>24.86</x:v>
       </x:c>
       <x:c r="J30" s="0">
         <x:v>21.09</x:v>
       </x:c>
       <x:c r="K30" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:11">
       <x:c r="A31" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C31" s="0">
         <x:v>201000</x:v>
@@ -2412,21 +2415,21 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>10.2</x:v>
+        <x:v>10.28</x:v>
       </x:c>
       <x:c r="J31" s="0">
         <x:v>10.31</x:v>
       </x:c>
       <x:c r="K31" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:11">
       <x:c r="A32" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
         <x:v>13</x:v>
@@ -2447,7 +2450,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I32" s="0">
-        <x:v>9.13</x:v>
+        <x:v>9.21</x:v>
       </x:c>
       <x:c r="J32" s="0">
         <x:v>0</x:v>
@@ -2455,10 +2458,10 @@
     </x:row>
     <x:row r="33" spans="1:11">
       <x:c r="A33" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C33" s="0">
         <x:v>1900000</x:v>
@@ -2479,21 +2482,21 @@
         <x:v>0.35</x:v>
       </x:c>
       <x:c r="I33" s="0">
-        <x:v>8.54</x:v>
+        <x:v>8.53</x:v>
       </x:c>
       <x:c r="J33" s="0">
         <x:v>7.46</x:v>
       </x:c>
       <x:c r="K33" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:11">
       <x:c r="A34" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="C34" s="0" t="s">
         <x:v>13</x:v>
@@ -2514,7 +2517,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I34" s="0">
-        <x:v>189.8</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="J34" s="0">
         <x:v>0</x:v>
@@ -2522,10 +2525,10 @@
     </x:row>
     <x:row r="35" spans="1:11">
       <x:c r="A35" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C35" s="0">
         <x:v>17879000</x:v>
@@ -2546,21 +2549,21 @@
         <x:v>0.82</x:v>
       </x:c>
       <x:c r="I35" s="0">
-        <x:v>19.05</x:v>
+        <x:v>18.59</x:v>
       </x:c>
       <x:c r="J35" s="0">
         <x:v>7.13</x:v>
       </x:c>
       <x:c r="K35" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:11">
       <x:c r="A36" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C36" s="0">
         <x:v>970810</x:v>
@@ -2581,21 +2584,21 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I36" s="0">
-        <x:v>22.96</x:v>
+        <x:v>22.92</x:v>
       </x:c>
       <x:c r="J36" s="0">
         <x:v>28.89</x:v>
       </x:c>
       <x:c r="K36" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:11">
       <x:c r="A37" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C37" s="0">
         <x:v>1001579</x:v>
@@ -2616,21 +2619,21 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I37" s="0">
-        <x:v>9.34</x:v>
+        <x:v>9.43</x:v>
       </x:c>
       <x:c r="J37" s="0">
         <x:v>15.08</x:v>
       </x:c>
       <x:c r="K37" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:11">
       <x:c r="A38" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C38" s="0" t="s">
         <x:v>13</x:v>
@@ -2651,7 +2654,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I38" s="0">
-        <x:v>4.55</x:v>
+        <x:v>4.68</x:v>
       </x:c>
       <x:c r="J38" s="0">
         <x:v>0</x:v>
@@ -2659,10 +2662,10 @@
     </x:row>
     <x:row r="39" spans="1:11">
       <x:c r="A39" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C39" s="0">
         <x:v>2097370</x:v>
@@ -2683,7 +2686,7 @@
         <x:v>2.78</x:v>
       </x:c>
       <x:c r="I39" s="0">
-        <x:v>20.08</x:v>
+        <x:v>21.82</x:v>
       </x:c>
       <x:c r="J39" s="0">
         <x:v>23.25</x:v>
@@ -2694,13 +2697,13 @@
     </x:row>
     <x:row r="40" spans="1:11">
       <x:c r="A40" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C40" s="0">
-        <x:v>28117493</x:v>
+        <x:v>28532493</x:v>
       </x:c>
       <x:c r="D40" s="0">
         <x:v>80000000</x:v>
@@ -2709,30 +2712,30 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F40" s="0">
-        <x:v>778677750</x:v>
+        <x:v>794742815</x:v>
       </x:c>
       <x:c r="G40" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H40" s="0">
-        <x:v>1.08</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="I40" s="0">
-        <x:v>38.36</x:v>
+        <x:v>38.42</x:v>
       </x:c>
       <x:c r="J40" s="0">
-        <x:v>27.69</x:v>
+        <x:v>27.85</x:v>
       </x:c>
       <x:c r="K40" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:11">
       <x:c r="A41" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C41" s="0">
         <x:v>7024156</x:v>
@@ -2753,21 +2756,21 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I41" s="0">
-        <x:v>11.31</x:v>
+        <x:v>11.29</x:v>
       </x:c>
       <x:c r="J41" s="0">
         <x:v>13.34</x:v>
       </x:c>
       <x:c r="K41" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:11">
       <x:c r="A42" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B42" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C42" s="0">
         <x:v>3500000</x:v>
@@ -2788,21 +2791,21 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I42" s="0">
-        <x:v>37.12</x:v>
+        <x:v>37.26</x:v>
       </x:c>
       <x:c r="J42" s="0">
         <x:v>39.18</x:v>
       </x:c>
       <x:c r="K42" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:11">
       <x:c r="A43" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="C43" s="0">
         <x:v>3753472</x:v>
@@ -2823,21 +2826,21 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="I43" s="0">
-        <x:v>61.5</x:v>
+        <x:v>61.45</x:v>
       </x:c>
       <x:c r="J43" s="0">
         <x:v>59.93</x:v>
       </x:c>
       <x:c r="K43" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:11">
       <x:c r="A44" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B44" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C44" s="0">
         <x:v>3189049</x:v>
@@ -2858,21 +2861,21 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="I44" s="0">
-        <x:v>5.8</x:v>
+        <x:v>5.69</x:v>
       </x:c>
       <x:c r="J44" s="0">
         <x:v>48.39</x:v>
       </x:c>
       <x:c r="K44" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:11">
       <x:c r="A45" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C45" s="0" t="s">
         <x:v>13</x:v>
@@ -2893,7 +2896,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I45" s="0">
-        <x:v>3.72</x:v>
+        <x:v>3.93</x:v>
       </x:c>
       <x:c r="J45" s="0">
         <x:v>0</x:v>
@@ -2901,10 +2904,10 @@
     </x:row>
     <x:row r="46" spans="1:11">
       <x:c r="A46" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C46" s="0">
         <x:v>3540000</x:v>
@@ -2925,7 +2928,7 @@
         <x:v>0.43</x:v>
       </x:c>
       <x:c r="I46" s="0">
-        <x:v>22.72</x:v>
+        <x:v>23.5</x:v>
       </x:c>
       <x:c r="J46" s="0">
         <x:v>45.09</x:v>
@@ -2936,13 +2939,13 @@
     </x:row>
     <x:row r="47" spans="1:11">
       <x:c r="A47" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C47" s="0">
-        <x:v>15525421</x:v>
+        <x:v>16715421</x:v>
       </x:c>
       <x:c r="D47" s="0">
         <x:v>35000000</x:v>
@@ -2951,30 +2954,30 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F47" s="0">
-        <x:v>133488395</x:v>
+        <x:v>145342995</x:v>
       </x:c>
       <x:c r="G47" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H47" s="0">
-        <x:v>3.88</x:v>
+        <x:v>4.18</x:v>
       </x:c>
       <x:c r="I47" s="0">
-        <x:v>9.63</x:v>
+        <x:v>9.42</x:v>
       </x:c>
       <x:c r="J47" s="0">
-        <x:v>8.6</x:v>
+        <x:v>8.7</x:v>
       </x:c>
       <x:c r="K47" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:11">
       <x:c r="A48" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B48" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="C48" s="0">
         <x:v>236122</x:v>
@@ -2995,21 +2998,21 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I48" s="0">
-        <x:v>78.8</x:v>
+        <x:v>77.8</x:v>
       </x:c>
       <x:c r="J48" s="0">
         <x:v>61.87</x:v>
       </x:c>
       <x:c r="K48" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:11">
       <x:c r="A49" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B49" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C49" s="0">
         <x:v>1000000</x:v>
@@ -3030,21 +3033,21 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I49" s="0">
-        <x:v>18.66</x:v>
+        <x:v>18.16</x:v>
       </x:c>
       <x:c r="J49" s="0">
         <x:v>21.06</x:v>
       </x:c>
       <x:c r="K49" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:11">
       <x:c r="A50" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B50" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C50" s="0" t="s">
         <x:v>13</x:v>
@@ -3065,7 +3068,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I50" s="0">
-        <x:v>5.8</x:v>
+        <x:v>5.69</x:v>
       </x:c>
       <x:c r="J50" s="0">
         <x:v>0</x:v>
@@ -3073,13 +3076,13 @@
     </x:row>
     <x:row r="51" spans="1:11">
       <x:c r="A51" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B51" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="C51" s="0">
-        <x:v>102967273</x:v>
+        <x:v>103967273</x:v>
       </x:c>
       <x:c r="D51" s="0">
         <x:v>200000000</x:v>
@@ -3088,30 +3091,30 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F51" s="0">
-        <x:v>1005509268</x:v>
+        <x:v>1016303268</x:v>
       </x:c>
       <x:c r="G51" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H51" s="0">
-        <x:v>1.14</x:v>
+        <x:v>1.16</x:v>
       </x:c>
       <x:c r="I51" s="0">
-        <x:v>10.82</x:v>
+        <x:v>11.09</x:v>
       </x:c>
       <x:c r="J51" s="0">
-        <x:v>9.77</x:v>
+        <x:v>9.78</x:v>
       </x:c>
       <x:c r="K51" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:11">
       <x:c r="A52" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B52" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C52" s="0">
         <x:v>16445115</x:v>
@@ -3138,15 +3141,15 @@
         <x:v>23.95</x:v>
       </x:c>
       <x:c r="K52" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:11">
       <x:c r="A53" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B53" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="C53" s="0">
         <x:v>1110000</x:v>
@@ -3167,21 +3170,21 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I53" s="0">
-        <x:v>420.5</x:v>
+        <x:v>427.5</x:v>
       </x:c>
       <x:c r="J53" s="0">
         <x:v>528.86</x:v>
       </x:c>
       <x:c r="K53" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:11">
       <x:c r="A54" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B54" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C54" s="0">
         <x:v>24398659</x:v>
@@ -3202,21 +3205,21 @@
         <x:v>0.94</x:v>
       </x:c>
       <x:c r="I54" s="0">
-        <x:v>38.36</x:v>
+        <x:v>38.42</x:v>
       </x:c>
       <x:c r="J54" s="0">
         <x:v>24.19</x:v>
       </x:c>
       <x:c r="K54" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:11">
       <x:c r="A55" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C55" s="0">
         <x:v>46563878</x:v>
@@ -3237,13 +3240,13 @@
         <x:v>0.52</x:v>
       </x:c>
       <x:c r="I55" s="0">
-        <x:v>10.82</x:v>
+        <x:v>11.09</x:v>
       </x:c>
       <x:c r="J55" s="0">
         <x:v>10.74</x:v>
       </x:c>
       <x:c r="K55" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:11">
@@ -3251,7 +3254,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
-        <x:v>128</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C56" s="0">
         <x:v>6611571</x:v>
@@ -3272,21 +3275,21 @@
         <x:v>0.69</x:v>
       </x:c>
       <x:c r="I56" s="0">
-        <x:v>6.91</x:v>
+        <x:v>6.65</x:v>
       </x:c>
       <x:c r="J56" s="0">
         <x:v>6.01</x:v>
       </x:c>
       <x:c r="K56" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:11">
       <x:c r="A57" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B57" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C57" s="0">
         <x:v>2596120</x:v>
@@ -3307,7 +3310,7 @@
         <x:v>1.36</x:v>
       </x:c>
       <x:c r="I57" s="0">
-        <x:v>19.2</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="J57" s="0">
         <x:v>25.45</x:v>
@@ -3318,10 +3321,10 @@
     </x:row>
     <x:row r="58" spans="1:11">
       <x:c r="A58" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B58" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C58" s="0">
         <x:v>1000000</x:v>
@@ -3342,13 +3345,13 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I58" s="0">
-        <x:v>3.79</x:v>
+        <x:v>3.74</x:v>
       </x:c>
       <x:c r="J58" s="0">
         <x:v>4.46</x:v>
       </x:c>
       <x:c r="K58" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:11">
@@ -3356,7 +3359,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C59" s="0">
         <x:v>200000</x:v>
@@ -3377,21 +3380,21 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I59" s="0">
-        <x:v>6.8</x:v>
+        <x:v>6.63</x:v>
       </x:c>
       <x:c r="J59" s="0">
         <x:v>12.82</x:v>
       </x:c>
       <x:c r="K59" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:11">
       <x:c r="A60" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B60" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="C60" s="0" t="s">
         <x:v>13</x:v>
@@ -3412,7 +3415,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I60" s="0">
-        <x:v>33.5</x:v>
+        <x:v>33.1</x:v>
       </x:c>
       <x:c r="J60" s="0">
         <x:v>0</x:v>
@@ -3420,10 +3423,10 @@
     </x:row>
     <x:row r="61" spans="1:11">
       <x:c r="A61" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B61" s="0" t="s">
-        <x:v>140</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C61" s="0">
         <x:v>5831653</x:v>
@@ -3444,21 +3447,21 @@
         <x:v>0.83</x:v>
       </x:c>
       <x:c r="I61" s="0">
-        <x:v>3</x:v>
+        <x:v>3.03</x:v>
       </x:c>
       <x:c r="J61" s="0">
         <x:v>52.14</x:v>
       </x:c>
       <x:c r="K61" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>142</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:11">
       <x:c r="A62" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B62" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="C62" s="0">
         <x:v>14512000</x:v>
@@ -3479,24 +3482,24 @@
         <x:v>1.83</x:v>
       </x:c>
       <x:c r="I62" s="0">
-        <x:v>36.62</x:v>
+        <x:v>36.7</x:v>
       </x:c>
       <x:c r="J62" s="0">
         <x:v>39.62</x:v>
       </x:c>
       <x:c r="K62" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>145</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:11">
       <x:c r="A63" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B63" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C63" s="0">
-        <x:v>3493291</x:v>
+        <x:v>3729828</x:v>
       </x:c>
       <x:c r="D63" s="0">
         <x:v>3000000</x:v>
@@ -3505,30 +3508,30 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F63" s="0">
-        <x:v>170794785</x:v>
+        <x:v>176220944</x:v>
       </x:c>
       <x:c r="G63" s="0">
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="H63" s="0">
-        <x:v>0.87</x:v>
+        <x:v>0.93</x:v>
       </x:c>
       <x:c r="I63" s="0">
-        <x:v>23.34</x:v>
+        <x:v>23.4</x:v>
       </x:c>
       <x:c r="J63" s="0">
-        <x:v>48.89</x:v>
+        <x:v>47.25</x:v>
       </x:c>
       <x:c r="K63" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:11">
       <x:c r="A64" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B64" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="C64" s="0" t="s">
         <x:v>13</x:v>
@@ -3549,7 +3552,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I64" s="0">
-        <x:v>26.18</x:v>
+        <x:v>26.02</x:v>
       </x:c>
       <x:c r="J64" s="0">
         <x:v>0</x:v>
@@ -3557,10 +3560,10 @@
     </x:row>
     <x:row r="65" spans="1:11">
       <x:c r="A65" s="0" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="B65" s="0" t="s">
         <x:v>149</x:v>
-      </x:c>
-      <x:c r="B65" s="0" t="s">
-        <x:v>148</x:v>
       </x:c>
       <x:c r="C65" s="0">
         <x:v>8337681</x:v>
@@ -3581,7 +3584,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I65" s="0">
-        <x:v>4.02</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="J65" s="0">
         <x:v>4.47</x:v>
@@ -3592,10 +3595,10 @@
     </x:row>
     <x:row r="66" spans="1:11">
       <x:c r="A66" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B66" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="C66" s="0" t="s">
         <x:v>13</x:v>
@@ -3616,7 +3619,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I66" s="0">
-        <x:v>40.2</x:v>
+        <x:v>39.94</x:v>
       </x:c>
       <x:c r="J66" s="0">
         <x:v>0</x:v>
@@ -3624,10 +3627,10 @@
     </x:row>
     <x:row r="67" spans="1:11">
       <x:c r="A67" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B67" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C67" s="0">
         <x:v>1364000</x:v>
@@ -3648,21 +3651,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I67" s="0">
-        <x:v>305</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="J67" s="0">
         <x:v>299.91</x:v>
       </x:c>
       <x:c r="K67" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:11">
       <x:c r="A68" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B68" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="C68" s="0" t="s">
         <x:v>13</x:v>
@@ -3683,7 +3686,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I68" s="0">
-        <x:v>20.44</x:v>
+        <x:v>22.48</x:v>
       </x:c>
       <x:c r="J68" s="0">
         <x:v>0</x:v>
@@ -3691,10 +3694,10 @@
     </x:row>
     <x:row r="69" spans="1:11">
       <x:c r="A69" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B69" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="C69" s="0">
         <x:v>507440</x:v>
@@ -3715,21 +3718,21 @@
         <x:v>0.54</x:v>
       </x:c>
       <x:c r="I69" s="0">
-        <x:v>294.5</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="J69" s="0">
         <x:v>83</x:v>
       </x:c>
       <x:c r="K69" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:11">
       <x:c r="A70" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B70" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C70" s="0">
         <x:v>2000000</x:v>
@@ -3750,13 +3753,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I70" s="0">
-        <x:v>34.76</x:v>
+        <x:v>35.18</x:v>
       </x:c>
       <x:c r="J70" s="0">
         <x:v>40.97</x:v>
       </x:c>
       <x:c r="K70" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="71" spans="1:11">
@@ -3764,7 +3767,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B71" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C71" s="0">
         <x:v>9854768</x:v>
@@ -3785,7 +3788,7 @@
         <x:v>0.62</x:v>
       </x:c>
       <x:c r="I71" s="0">
-        <x:v>21.34</x:v>
+        <x:v>21.18</x:v>
       </x:c>
       <x:c r="J71" s="0">
         <x:v>23.68</x:v>
@@ -3796,10 +3799,10 @@
     </x:row>
     <x:row r="72" spans="1:11">
       <x:c r="A72" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B72" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C72" s="0">
         <x:v>324474</x:v>
@@ -3820,13 +3823,13 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I72" s="0">
-        <x:v>15.94</x:v>
+        <x:v>16.43</x:v>
       </x:c>
       <x:c r="J72" s="0">
         <x:v>5.49</x:v>
       </x:c>
       <x:c r="K72" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="73" spans="1:11">
@@ -3834,7 +3837,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B73" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C73" s="0" t="s">
         <x:v>13</x:v>
@@ -3855,7 +3858,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I73" s="0">
-        <x:v>18.13</x:v>
+        <x:v>16.52</x:v>
       </x:c>
       <x:c r="J73" s="0">
         <x:v>0</x:v>
@@ -3863,10 +3866,10 @@
     </x:row>
     <x:row r="74" spans="1:11">
       <x:c r="A74" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B74" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="C74" s="0" t="s">
         <x:v>13</x:v>
@@ -3887,7 +3890,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I74" s="0">
-        <x:v>5.33</x:v>
+        <x:v>5.38</x:v>
       </x:c>
       <x:c r="J74" s="0">
         <x:v>0</x:v>
@@ -3895,10 +3898,10 @@
     </x:row>
     <x:row r="75" spans="1:11">
       <x:c r="A75" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B75" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="C75" s="0">
         <x:v>13000000</x:v>
@@ -3919,21 +3922,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I75" s="0">
-        <x:v>6.58</x:v>
+        <x:v>6.66</x:v>
       </x:c>
       <x:c r="J75" s="0">
         <x:v>6.6</x:v>
       </x:c>
       <x:c r="K75" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="76" spans="1:11">
       <x:c r="A76" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B76" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="C76" s="0">
         <x:v>174500000</x:v>
@@ -3954,21 +3957,21 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I76" s="0">
-        <x:v>2.76</x:v>
+        <x:v>2.73</x:v>
       </x:c>
       <x:c r="J76" s="0">
         <x:v>3.98</x:v>
       </x:c>
       <x:c r="K76" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="77" spans="1:11">
       <x:c r="A77" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B77" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C77" s="0">
         <x:v>635229</x:v>
@@ -3989,21 +3992,21 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I77" s="0">
-        <x:v>19.2</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="J77" s="0">
         <x:v>17.83</x:v>
       </x:c>
       <x:c r="K77" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="78" spans="1:11">
       <x:c r="A78" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B78" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="C78" s="0">
         <x:v>130000</x:v>
@@ -4024,21 +4027,21 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I78" s="0">
-        <x:v>29.44</x:v>
+        <x:v>29.5</x:v>
       </x:c>
       <x:c r="J78" s="0">
         <x:v>38.06</x:v>
       </x:c>
       <x:c r="K78" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="79" spans="1:11">
       <x:c r="A79" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B79" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="C79" s="0" t="s">
         <x:v>13</x:v>
@@ -4059,7 +4062,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I79" s="0">
-        <x:v>221.8</x:v>
+        <x:v>220.9</x:v>
       </x:c>
       <x:c r="J79" s="0">
         <x:v>0</x:v>
@@ -4067,10 +4070,10 @@
     </x:row>
     <x:row r="80" spans="1:11">
       <x:c r="A80" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B80" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C80" s="0">
         <x:v>447761</x:v>
@@ -4091,21 +4094,21 @@
         <x:v>0.86</x:v>
       </x:c>
       <x:c r="I80" s="0">
-        <x:v>34.02</x:v>
+        <x:v>34.3</x:v>
       </x:c>
       <x:c r="J80" s="0">
         <x:v>41.13</x:v>
       </x:c>
       <x:c r="K80" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="81" spans="1:11">
       <x:c r="A81" s="0" t="s">
-        <x:v>179</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="B81" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C81" s="0">
         <x:v>200000</x:v>
@@ -4126,21 +4129,21 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I81" s="0">
-        <x:v>4.66</x:v>
+        <x:v>4.63</x:v>
       </x:c>
       <x:c r="J81" s="0">
         <x:v>20.11</x:v>
       </x:c>
       <x:c r="K81" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="82" spans="1:11">
       <x:c r="A82" s="0" t="s">
-        <x:v>182</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B82" s="0" t="s">
-        <x:v>183</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C82" s="0">
         <x:v>946718</x:v>
@@ -4161,21 +4164,21 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I82" s="0">
-        <x:v>47.3</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="J82" s="0">
         <x:v>39.43</x:v>
       </x:c>
       <x:c r="K82" s="0" t="s">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
     </x:row>
     <x:row r="83" spans="1:11">
       <x:c r="A83" s="0" t="s">
-        <x:v>185</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="B83" s="0" t="s">
-        <x:v>186</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="C83" s="0" t="s">
         <x:v>13</x:v>
@@ -4196,7 +4199,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I83" s="0">
-        <x:v>19.01</x:v>
+        <x:v>18.58</x:v>
       </x:c>
       <x:c r="J83" s="0">
         <x:v>0</x:v>
@@ -4204,10 +4207,10 @@
     </x:row>
     <x:row r="84" spans="1:11">
       <x:c r="A84" s="0" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="B84" s="0" t="s">
         <x:v>187</x:v>
-      </x:c>
-      <x:c r="B84" s="0" t="s">
-        <x:v>186</x:v>
       </x:c>
       <x:c r="C84" s="0">
         <x:v>3043115</x:v>
@@ -4228,21 +4231,21 @@
         <x:v>0.12</x:v>
       </x:c>
       <x:c r="I84" s="0">
-        <x:v>21.76</x:v>
+        <x:v>21.5</x:v>
       </x:c>
       <x:c r="J84" s="0">
         <x:v>16.34</x:v>
       </x:c>
       <x:c r="K84" s="0" t="s">
-        <x:v>188</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="85" spans="1:11">
       <x:c r="A85" s="0" t="s">
-        <x:v>189</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B85" s="0" t="s">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C85" s="0">
         <x:v>2382736</x:v>
@@ -4263,21 +4266,21 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="I85" s="0">
-        <x:v>71.05</x:v>
+        <x:v>72.6</x:v>
       </x:c>
       <x:c r="J85" s="0">
         <x:v>38.88</x:v>
       </x:c>
       <x:c r="K85" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="86" spans="1:11">
       <x:c r="A86" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="B86" s="0" t="s">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C86" s="0" t="s">
         <x:v>13</x:v>
@@ -4298,7 +4301,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I86" s="0">
-        <x:v>53</x:v>
+        <x:v>51.3</x:v>
       </x:c>
       <x:c r="J86" s="0">
         <x:v>0</x:v>
@@ -4306,10 +4309,10 @@
     </x:row>
     <x:row r="87" spans="1:11">
       <x:c r="A87" s="0" t="s">
-        <x:v>193</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B87" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="C87" s="0">
         <x:v>4650000</x:v>
@@ -4330,21 +4333,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I87" s="0">
-        <x:v>11.64</x:v>
+        <x:v>12.34</x:v>
       </x:c>
       <x:c r="J87" s="0">
         <x:v>10.75</x:v>
       </x:c>
       <x:c r="K87" s="0" t="s">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="88" spans="1:11">
       <x:c r="A88" s="0" t="s">
-        <x:v>196</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B88" s="0" t="s">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C88" s="0">
         <x:v>806343</x:v>
@@ -4365,7 +4368,7 @@
         <x:v>2.16</x:v>
       </x:c>
       <x:c r="I88" s="0">
-        <x:v>34.18</x:v>
+        <x:v>34.3</x:v>
       </x:c>
       <x:c r="J88" s="0">
         <x:v>37.66</x:v>
@@ -4376,10 +4379,10 @@
     </x:row>
     <x:row r="89" spans="1:11">
       <x:c r="A89" s="0" t="s">
-        <x:v>193</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B89" s="0" t="s">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C89" s="0">
         <x:v>310000</x:v>
@@ -4400,13 +4403,13 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I89" s="0">
-        <x:v>11.64</x:v>
+        <x:v>12.34</x:v>
       </x:c>
       <x:c r="J89" s="0">
         <x:v>161.23</x:v>
       </x:c>
       <x:c r="K89" s="0" t="s">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="90" spans="1:11">
@@ -4414,7 +4417,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B90" s="0" t="s">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C90" s="0">
         <x:v>2000000</x:v>
@@ -4435,21 +4438,21 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="I90" s="0">
-        <x:v>9.15</x:v>
+        <x:v>9.23</x:v>
       </x:c>
       <x:c r="J90" s="0">
         <x:v>15.68</x:v>
       </x:c>
       <x:c r="K90" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="91" spans="1:11">
       <x:c r="A91" s="0" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="B91" s="0" t="s">
         <x:v>198</x:v>
-      </x:c>
-      <x:c r="B91" s="0" t="s">
-        <x:v>197</x:v>
       </x:c>
       <x:c r="C91" s="0">
         <x:v>1250000</x:v>
@@ -4476,15 +4479,15 @@
         <x:v>8.95</x:v>
       </x:c>
       <x:c r="K91" s="0" t="s">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="92" spans="1:11">
       <x:c r="A92" s="0" t="s">
-        <x:v>199</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B92" s="0" t="s">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C92" s="0" t="s">
         <x:v>13</x:v>
@@ -4505,7 +4508,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I92" s="0">
-        <x:v>4.01</x:v>
+        <x:v>3.99</x:v>
       </x:c>
       <x:c r="J92" s="0">
         <x:v>0</x:v>
@@ -4513,10 +4516,10 @@
     </x:row>
     <x:row r="93" spans="1:11">
       <x:c r="A93" s="0" t="s">
-        <x:v>200</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B93" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C93" s="0">
         <x:v>12500000</x:v>
@@ -4537,21 +4540,21 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="I93" s="0">
-        <x:v>2.09</x:v>
+        <x:v>2.08</x:v>
       </x:c>
       <x:c r="J93" s="0">
         <x:v>4.93</x:v>
       </x:c>
       <x:c r="K93" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="94" spans="1:11">
       <x:c r="A94" s="0" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="B94" s="0" t="s">
         <x:v>202</x:v>
-      </x:c>
-      <x:c r="B94" s="0" t="s">
-        <x:v>201</x:v>
       </x:c>
       <x:c r="C94" s="0">
         <x:v>2093944</x:v>
@@ -4572,21 +4575,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I94" s="0">
-        <x:v>101.6</x:v>
+        <x:v>101.8</x:v>
       </x:c>
       <x:c r="J94" s="0">
         <x:v>95.58</x:v>
       </x:c>
       <x:c r="K94" s="0" t="s">
-        <x:v>203</x:v>
+        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="95" spans="1:11">
       <x:c r="A95" s="0" t="s">
-        <x:v>204</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="B95" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C95" s="0" t="s">
         <x:v>13</x:v>
@@ -4607,7 +4610,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I95" s="0">
-        <x:v>50.8</x:v>
+        <x:v>50.2</x:v>
       </x:c>
       <x:c r="J95" s="0">
         <x:v>0</x:v>
@@ -4615,10 +4618,10 @@
     </x:row>
     <x:row r="96" spans="1:11">
       <x:c r="A96" s="0" t="s">
-        <x:v>205</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="B96" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C96" s="0">
         <x:v>51245979</x:v>
@@ -4639,13 +4642,13 @@
         <x:v>1.31</x:v>
       </x:c>
       <x:c r="I96" s="0">
-        <x:v>2.58</x:v>
+        <x:v>2.61</x:v>
       </x:c>
       <x:c r="J96" s="0">
         <x:v>2.45</x:v>
       </x:c>
       <x:c r="K96" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="97" spans="1:11">
@@ -4653,7 +4656,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B97" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C97" s="0">
         <x:v>1584837</x:v>
@@ -4674,21 +4677,21 @@
         <x:v>1.08</x:v>
       </x:c>
       <x:c r="I97" s="0">
-        <x:v>67.3</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="J97" s="0">
         <x:v>58.33</x:v>
       </x:c>
       <x:c r="K97" s="0" t="s">
-        <x:v>206</x:v>
+        <x:v>207</x:v>
       </x:c>
     </x:row>
     <x:row r="98" spans="1:11">
       <x:c r="A98" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B98" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C98" s="0">
         <x:v>7999148</x:v>
@@ -4709,21 +4712,21 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I98" s="0">
-        <x:v>24.18</x:v>
+        <x:v>24.86</x:v>
       </x:c>
       <x:c r="J98" s="0">
         <x:v>21.09</x:v>
       </x:c>
       <x:c r="K98" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="99" spans="1:11">
       <x:c r="A99" s="0" t="s">
-        <x:v>207</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="B99" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C99" s="0">
         <x:v>14000000</x:v>
@@ -4744,13 +4747,13 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I99" s="0">
-        <x:v>24.1</x:v>
+        <x:v>26.5</x:v>
       </x:c>
       <x:c r="J99" s="0">
         <x:v>16.87</x:v>
       </x:c>
       <x:c r="K99" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="100" spans="1:11">
@@ -4758,7 +4761,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B100" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C100" s="0">
         <x:v>1700005</x:v>
@@ -4779,21 +4782,21 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I100" s="0">
-        <x:v>5.59</x:v>
+        <x:v>5.54</x:v>
       </x:c>
       <x:c r="J100" s="0">
         <x:v>11.99</x:v>
       </x:c>
       <x:c r="K100" s="0" t="s">
-        <x:v>208</x:v>
+        <x:v>209</x:v>
       </x:c>
     </x:row>
     <x:row r="101" spans="1:11">
       <x:c r="A101" s="0" t="s">
-        <x:v>209</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="B101" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C101" s="0">
         <x:v>6000000</x:v>
@@ -4814,21 +4817,21 @@
         <x:v>0.16</x:v>
       </x:c>
       <x:c r="I101" s="0">
-        <x:v>17.53</x:v>
+        <x:v>17.27</x:v>
       </x:c>
       <x:c r="J101" s="0">
         <x:v>22.05</x:v>
       </x:c>
       <x:c r="K101" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="102" spans="1:11">
       <x:c r="A102" s="0" t="s">
-        <x:v>212</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="B102" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C102" s="0">
         <x:v>1675000</x:v>
@@ -4849,21 +4852,21 @@
         <x:v>1.45</x:v>
       </x:c>
       <x:c r="I102" s="0">
-        <x:v>87.9</x:v>
+        <x:v>86.05</x:v>
       </x:c>
       <x:c r="J102" s="0">
         <x:v>68.15</x:v>
       </x:c>
       <x:c r="K102" s="0" t="s">
-        <x:v>213</x:v>
+        <x:v>214</x:v>
       </x:c>
     </x:row>
     <x:row r="103" spans="1:11">
       <x:c r="A103" s="0" t="s">
-        <x:v>214</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="B103" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C103" s="0">
         <x:v>1824868</x:v>
@@ -4884,7 +4887,7 @@
         <x:v>0.68</x:v>
       </x:c>
       <x:c r="I103" s="0">
-        <x:v>31</x:v>
+        <x:v>30.8</x:v>
       </x:c>
       <x:c r="J103" s="0">
         <x:v>35.38</x:v>
@@ -4895,10 +4898,10 @@
     </x:row>
     <x:row r="104" spans="1:11">
       <x:c r="A104" s="0" t="s">
-        <x:v>215</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B104" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C104" s="0" t="s">
         <x:v>13</x:v>
@@ -4919,7 +4922,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I104" s="0">
-        <x:v>6.88</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="J104" s="0">
         <x:v>0</x:v>
@@ -4927,10 +4930,10 @@
     </x:row>
     <x:row r="105" spans="1:11">
       <x:c r="A105" s="0" t="s">
-        <x:v>216</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B105" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C105" s="0">
         <x:v>1000000</x:v>
@@ -4951,21 +4954,21 @@
         <x:v>0.27</x:v>
       </x:c>
       <x:c r="I105" s="0">
-        <x:v>9.49</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="J105" s="0">
         <x:v>19.79</x:v>
       </x:c>
       <x:c r="K105" s="0" t="s">
-        <x:v>217</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
     <x:row r="106" spans="1:11">
       <x:c r="A106" s="0" t="s">
-        <x:v>218</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B106" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C106" s="0">
         <x:v>98551</x:v>
@@ -4986,21 +4989,21 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I106" s="0">
-        <x:v>10.64</x:v>
+        <x:v>10.77</x:v>
       </x:c>
       <x:c r="J106" s="0">
         <x:v>13.15</x:v>
       </x:c>
       <x:c r="K106" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="107" spans="1:11">
       <x:c r="A107" s="0" t="s">
-        <x:v>219</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B107" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C107" s="0">
         <x:v>6049315</x:v>
@@ -5021,13 +5024,13 @@
         <x:v>0.92</x:v>
       </x:c>
       <x:c r="I107" s="0">
-        <x:v>11.31</x:v>
+        <x:v>11.37</x:v>
       </x:c>
       <x:c r="J107" s="0">
         <x:v>10.98</x:v>
       </x:c>
       <x:c r="K107" s="0" t="s">
-        <x:v>220</x:v>
+        <x:v>221</x:v>
       </x:c>
     </x:row>
     <x:row r="108" spans="1:11">
@@ -5035,7 +5038,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B108" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C108" s="0">
         <x:v>37225000</x:v>
@@ -5056,21 +5059,21 @@
         <x:v>3.45</x:v>
       </x:c>
       <x:c r="I108" s="0">
-        <x:v>1.68</x:v>
+        <x:v>1.7</x:v>
       </x:c>
       <x:c r="J108" s="0">
         <x:v>4.03</x:v>
       </x:c>
       <x:c r="K108" s="0" t="s">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="109" spans="1:11">
       <x:c r="A109" s="0" t="s">
-        <x:v>221</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="B109" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C109" s="0">
         <x:v>1000000</x:v>
@@ -5091,21 +5094,21 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="I109" s="0">
-        <x:v>191.5</x:v>
+        <x:v>199.5</x:v>
       </x:c>
       <x:c r="J109" s="0">
         <x:v>284.58</x:v>
       </x:c>
       <x:c r="K109" s="0" t="s">
-        <x:v>222</x:v>
+        <x:v>223</x:v>
       </x:c>
     </x:row>
     <x:row r="110" spans="1:11">
       <x:c r="A110" s="0" t="s">
-        <x:v>223</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="B110" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C110" s="0">
         <x:v>600000</x:v>
@@ -5126,21 +5129,21 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="I110" s="0">
-        <x:v>6.04</x:v>
+        <x:v>5.88</x:v>
       </x:c>
       <x:c r="J110" s="0">
         <x:v>38.02</x:v>
       </x:c>
       <x:c r="K110" s="0" t="s">
-        <x:v>224</x:v>
+        <x:v>225</x:v>
       </x:c>
     </x:row>
     <x:row r="111" spans="1:11">
       <x:c r="A111" s="0" t="s">
-        <x:v>225</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="B111" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C111" s="0">
         <x:v>11703083</x:v>
@@ -5161,21 +5164,21 @@
         <x:v>1.67</x:v>
       </x:c>
       <x:c r="I111" s="0">
-        <x:v>195.5</x:v>
+        <x:v>195.6</x:v>
       </x:c>
       <x:c r="J111" s="0">
         <x:v>83.62</x:v>
       </x:c>
       <x:c r="K111" s="0" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
     </x:row>
     <x:row r="112" spans="1:11">
       <x:c r="A112" s="0" t="s">
-        <x:v>227</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B112" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C112" s="0">
         <x:v>5100000</x:v>
@@ -5196,13 +5199,13 @@
         <x:v>4.31</x:v>
       </x:c>
       <x:c r="I112" s="0">
-        <x:v>31.44</x:v>
+        <x:v>30.7</x:v>
       </x:c>
       <x:c r="J112" s="0">
         <x:v>17.65</x:v>
       </x:c>
       <x:c r="K112" s="0" t="s">
-        <x:v>228</x:v>
+        <x:v>229</x:v>
       </x:c>
     </x:row>
     <x:row r="113" spans="1:11">
@@ -5210,7 +5213,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B113" s="0" t="s">
-        <x:v>229</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C113" s="0">
         <x:v>3228679</x:v>
@@ -5231,21 +5234,21 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I113" s="0">
-        <x:v>8.6</x:v>
+        <x:v>8.94</x:v>
       </x:c>
       <x:c r="J113" s="0">
         <x:v>15.92</x:v>
       </x:c>
       <x:c r="K113" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="114" spans="1:11">
       <x:c r="A114" s="0" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="B114" s="0" t="s">
         <x:v>230</x:v>
-      </x:c>
-      <x:c r="B114" s="0" t="s">
-        <x:v>229</x:v>
       </x:c>
       <x:c r="C114" s="0">
         <x:v>150000</x:v>
@@ -5266,21 +5269,21 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I114" s="0">
-        <x:v>5.3</x:v>
+        <x:v>5.31</x:v>
       </x:c>
       <x:c r="J114" s="0">
         <x:v>40.97</x:v>
       </x:c>
       <x:c r="K114" s="0" t="s">
-        <x:v>231</x:v>
+        <x:v>232</x:v>
       </x:c>
     </x:row>
     <x:row r="115" spans="1:11">
       <x:c r="A115" s="0" t="s">
-        <x:v>232</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="B115" s="0" t="s">
-        <x:v>229</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C115" s="0" t="s">
         <x:v>13</x:v>
@@ -5301,7 +5304,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I115" s="0">
-        <x:v>10.44</x:v>
+        <x:v>10.17</x:v>
       </x:c>
       <x:c r="J115" s="0">
         <x:v>0</x:v>
@@ -5309,10 +5312,10 @@
     </x:row>
     <x:row r="116" spans="1:11">
       <x:c r="A116" s="0" t="s">
-        <x:v>233</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="B116" s="0" t="s">
-        <x:v>229</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C116" s="0">
         <x:v>366107</x:v>
@@ -5333,21 +5336,21 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I116" s="0">
-        <x:v>14.83</x:v>
+        <x:v>15.02</x:v>
       </x:c>
       <x:c r="J116" s="0">
         <x:v>16.42</x:v>
       </x:c>
       <x:c r="K116" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="117" spans="1:11">
       <x:c r="A117" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B117" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C117" s="0">
         <x:v>120000</x:v>
@@ -5368,21 +5371,21 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I117" s="0">
-        <x:v>189.8</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="J117" s="0">
         <x:v>31.92</x:v>
       </x:c>
       <x:c r="K117" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
     </x:row>
     <x:row r="118" spans="1:11">
       <x:c r="A118" s="0" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="B118" s="0" t="s">
         <x:v>235</x:v>
-      </x:c>
-      <x:c r="B118" s="0" t="s">
-        <x:v>234</x:v>
       </x:c>
       <x:c r="C118" s="0">
         <x:v>13050000</x:v>
@@ -5403,21 +5406,21 @@
         <x:v>3.13</x:v>
       </x:c>
       <x:c r="I118" s="0">
-        <x:v>115</x:v>
+        <x:v>116.3</x:v>
       </x:c>
       <x:c r="J118" s="0">
         <x:v>94.36</x:v>
       </x:c>
       <x:c r="K118" s="0" t="s">
-        <x:v>236</x:v>
+        <x:v>237</x:v>
       </x:c>
     </x:row>
     <x:row r="119" spans="1:11">
       <x:c r="A119" s="0" t="s">
-        <x:v>237</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="B119" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C119" s="0">
         <x:v>36605658</x:v>
@@ -5438,7 +5441,7 @@
         <x:v>3.66</x:v>
       </x:c>
       <x:c r="I119" s="0">
-        <x:v>4.79</x:v>
+        <x:v>4.69</x:v>
       </x:c>
       <x:c r="J119" s="0">
         <x:v>4.76</x:v>
@@ -5449,10 +5452,10 @@
     </x:row>
     <x:row r="120" spans="1:11">
       <x:c r="A120" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B120" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C120" s="0">
         <x:v>1000000</x:v>
@@ -5473,21 +5476,21 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I120" s="0">
-        <x:v>420.5</x:v>
+        <x:v>427.5</x:v>
       </x:c>
       <x:c r="J120" s="0">
         <x:v>429.82</x:v>
       </x:c>
       <x:c r="K120" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
     </x:row>
     <x:row r="121" spans="1:11">
       <x:c r="A121" s="0" t="s">
-        <x:v>238</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="B121" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C121" s="0">
         <x:v>300000</x:v>
@@ -5514,15 +5517,15 @@
         <x:v>2.64</x:v>
       </x:c>
       <x:c r="K121" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
     </x:row>
     <x:row r="122" spans="1:11">
       <x:c r="A122" s="0" t="s">
-        <x:v>239</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="B122" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C122" s="0">
         <x:v>2175097</x:v>
@@ -5549,15 +5552,15 @@
         <x:v>8.23</x:v>
       </x:c>
       <x:c r="K122" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="123" spans="1:11">
       <x:c r="A123" s="0" t="s">
-        <x:v>240</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="B123" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C123" s="0" t="s">
         <x:v>13</x:v>
@@ -5578,7 +5581,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I123" s="0">
-        <x:v>2.82</x:v>
+        <x:v>2.84</x:v>
       </x:c>
       <x:c r="J123" s="0">
         <x:v>0</x:v>
@@ -5586,10 +5589,10 @@
     </x:row>
     <x:row r="124" spans="1:11">
       <x:c r="A124" s="0" t="s">
-        <x:v>241</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="B124" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C124" s="0">
         <x:v>43000</x:v>
@@ -5610,21 +5613,21 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I124" s="0">
-        <x:v>28.12</x:v>
+        <x:v>27.6</x:v>
       </x:c>
       <x:c r="J124" s="0">
         <x:v>23.83</x:v>
       </x:c>
       <x:c r="K124" s="0" t="s">
-        <x:v>242</x:v>
+        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="125" spans="1:11">
       <x:c r="A125" s="0" t="s">
-        <x:v>243</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="B125" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C125" s="0">
         <x:v>9937037</x:v>
@@ -5645,21 +5648,21 @@
         <x:v>0.53</x:v>
       </x:c>
       <x:c r="I125" s="0">
-        <x:v>2.24</x:v>
+        <x:v>2.25</x:v>
       </x:c>
       <x:c r="J125" s="0">
         <x:v>5.03</x:v>
       </x:c>
       <x:c r="K125" s="0" t="s">
-        <x:v>244</x:v>
+        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="126" spans="1:11">
       <x:c r="A126" s="0" t="s">
-        <x:v>245</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="B126" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C126" s="0" t="s">
         <x:v>13</x:v>
@@ -5688,10 +5691,10 @@
     </x:row>
     <x:row r="127" spans="1:11">
       <x:c r="A127" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B127" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C127" s="0">
         <x:v>13064888</x:v>
@@ -5712,21 +5715,21 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I127" s="0">
-        <x:v>38.36</x:v>
+        <x:v>38.42</x:v>
       </x:c>
       <x:c r="J127" s="0">
         <x:v>20.53</x:v>
       </x:c>
       <x:c r="K127" s="0" t="s">
-        <x:v>246</x:v>
+        <x:v>247</x:v>
       </x:c>
     </x:row>
     <x:row r="128" spans="1:11">
       <x:c r="A128" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B128" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C128" s="0">
         <x:v>111673026</x:v>
@@ -5747,21 +5750,21 @@
         <x:v>1.24</x:v>
       </x:c>
       <x:c r="I128" s="0">
-        <x:v>10.82</x:v>
+        <x:v>11.09</x:v>
       </x:c>
       <x:c r="J128" s="0">
         <x:v>4.48</x:v>
       </x:c>
       <x:c r="K128" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="129" spans="1:11">
       <x:c r="A129" s="0" t="s">
-        <x:v>248</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B129" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C129" s="0" t="s">
         <x:v>13</x:v>
@@ -5782,7 +5785,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I129" s="0">
-        <x:v>3.74</x:v>
+        <x:v>3.71</x:v>
       </x:c>
       <x:c r="J129" s="0">
         <x:v>0</x:v>
@@ -5790,10 +5793,10 @@
     </x:row>
     <x:row r="130" spans="1:11">
       <x:c r="A130" s="0" t="s">
-        <x:v>249</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="B130" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C130" s="0" t="s">
         <x:v>13</x:v>
@@ -5814,7 +5817,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I130" s="0">
-        <x:v>7.17</x:v>
+        <x:v>7.09</x:v>
       </x:c>
       <x:c r="J130" s="0">
         <x:v>0</x:v>
@@ -5822,10 +5825,10 @@
     </x:row>
     <x:row r="131" spans="1:11">
       <x:c r="A131" s="0" t="s">
-        <x:v>250</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="B131" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C131" s="0">
         <x:v>1100000</x:v>
@@ -5846,13 +5849,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I131" s="0">
-        <x:v>164.2</x:v>
+        <x:v>154.2</x:v>
       </x:c>
       <x:c r="J131" s="0">
         <x:v>50.97</x:v>
       </x:c>
       <x:c r="K131" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="132" spans="1:11">
@@ -5860,7 +5863,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B132" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C132" s="0">
         <x:v>6598092</x:v>
@@ -5881,7 +5884,7 @@
         <x:v>5.91</x:v>
       </x:c>
       <x:c r="I132" s="0">
-        <x:v>18.13</x:v>
+        <x:v>16.52</x:v>
       </x:c>
       <x:c r="J132" s="0">
         <x:v>10.93</x:v>
@@ -5892,10 +5895,10 @@
     </x:row>
     <x:row r="133" spans="1:11">
       <x:c r="A133" s="0" t="s">
-        <x:v>251</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="B133" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C133" s="0">
         <x:v>1590000</x:v>
@@ -5916,21 +5919,21 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="I133" s="0">
-        <x:v>37.9</x:v>
+        <x:v>38.2</x:v>
       </x:c>
       <x:c r="J133" s="0">
         <x:v>38.14</x:v>
       </x:c>
       <x:c r="K133" s="0" t="s">
-        <x:v>252</x:v>
+        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="134" spans="1:11">
       <x:c r="A134" s="0" t="s">
-        <x:v>253</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="B134" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C134" s="0">
         <x:v>1989802</x:v>
@@ -5951,21 +5954,21 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I134" s="0">
-        <x:v>140.2</x:v>
+        <x:v>139.5</x:v>
       </x:c>
       <x:c r="J134" s="0">
         <x:v>39.56</x:v>
       </x:c>
       <x:c r="K134" s="0" t="s">
-        <x:v>254</x:v>
+        <x:v>255</x:v>
       </x:c>
     </x:row>
     <x:row r="135" spans="1:11">
       <x:c r="A135" s="0" t="s">
-        <x:v>255</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="B135" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C135" s="0" t="s">
         <x:v>13</x:v>
@@ -5986,7 +5989,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I135" s="0">
-        <x:v>510</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="J135" s="0">
         <x:v>0</x:v>
@@ -5994,10 +5997,10 @@
     </x:row>
     <x:row r="136" spans="1:11">
       <x:c r="A136" s="0" t="s">
-        <x:v>256</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B136" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C136" s="0">
         <x:v>300000</x:v>
@@ -6018,21 +6021,21 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I136" s="0">
-        <x:v>7.48</x:v>
+        <x:v>7.33</x:v>
       </x:c>
       <x:c r="J136" s="0">
         <x:v>4.56</x:v>
       </x:c>
       <x:c r="K136" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
     </x:row>
     <x:row r="137" spans="1:11">
       <x:c r="A137" s="0" t="s">
-        <x:v>257</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="B137" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C137" s="0">
         <x:v>76908759</x:v>
@@ -6053,21 +6056,21 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I137" s="0">
-        <x:v>36.64</x:v>
+        <x:v>35.52</x:v>
       </x:c>
       <x:c r="J137" s="0">
         <x:v>25.74</x:v>
       </x:c>
       <x:c r="K137" s="0" t="s">
-        <x:v>258</x:v>
+        <x:v>259</x:v>
       </x:c>
     </x:row>
     <x:row r="138" spans="1:11">
       <x:c r="A138" s="0" t="s">
-        <x:v>259</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="B138" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="C138" s="0">
         <x:v>8291656</x:v>
@@ -6088,21 +6091,21 @@
         <x:v>1.9</x:v>
       </x:c>
       <x:c r="I138" s="0">
-        <x:v>17.28</x:v>
+        <x:v>17.17</x:v>
       </x:c>
       <x:c r="J138" s="0">
         <x:v>15.2</x:v>
       </x:c>
       <x:c r="K138" s="0" t="s">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
     </x:row>
     <x:row r="139" spans="1:11">
       <x:c r="A139" s="0" t="s">
-        <x:v>260</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="B139" s="0" t="s">
-        <x:v>261</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="C139" s="0">
         <x:v>2975773</x:v>
@@ -6123,21 +6126,21 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="I139" s="0">
-        <x:v>26.34</x:v>
+        <x:v>26.22</x:v>
       </x:c>
       <x:c r="J139" s="0">
         <x:v>15.05</x:v>
       </x:c>
       <x:c r="K139" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="140" spans="1:11">
       <x:c r="A140" s="0" t="s">
-        <x:v>262</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="B140" s="0" t="s">
-        <x:v>263</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="C140" s="0">
         <x:v>10994323</x:v>
@@ -6158,21 +6161,21 @@
         <x:v>5.09</x:v>
       </x:c>
       <x:c r="I140" s="0">
-        <x:v>12.99</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="J140" s="0">
         <x:v>16.65</x:v>
       </x:c>
       <x:c r="K140" s="0" t="s">
-        <x:v>264</x:v>
+        <x:v>265</x:v>
       </x:c>
     </x:row>
     <x:row r="141" spans="1:11">
       <x:c r="A141" s="0" t="s">
-        <x:v>265</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="B141" s="0" t="s">
-        <x:v>266</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="C141" s="0">
         <x:v>36870641</x:v>
@@ -6193,7 +6196,7 @@
         <x:v>1.89</x:v>
       </x:c>
       <x:c r="I141" s="0">
-        <x:v>16.95</x:v>
+        <x:v>16.63</x:v>
       </x:c>
       <x:c r="J141" s="0">
         <x:v>11.29</x:v>
@@ -6204,10 +6207,10 @@
     </x:row>
     <x:row r="142" spans="1:11">
       <x:c r="A142" s="0" t="s">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="B142" s="0" t="s">
         <x:v>267</x:v>
-      </x:c>
-      <x:c r="B142" s="0" t="s">
-        <x:v>266</x:v>
       </x:c>
       <x:c r="C142" s="0">
         <x:v>5100000</x:v>
@@ -6228,21 +6231,21 @@
         <x:v>0.93</x:v>
       </x:c>
       <x:c r="I142" s="0">
-        <x:v>59.25</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="J142" s="0">
         <x:v>30.45</x:v>
       </x:c>
       <x:c r="K142" s="0" t="s">
-        <x:v>268</x:v>
+        <x:v>269</x:v>
       </x:c>
     </x:row>
     <x:row r="143" spans="1:11">
       <x:c r="A143" s="0" t="s">
-        <x:v>269</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="B143" s="0" t="s">
-        <x:v>270</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="C143" s="0" t="s">
         <x:v>13</x:v>
@@ -6263,7 +6266,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I143" s="0">
-        <x:v>2.05</x:v>
+        <x:v>2.09</x:v>
       </x:c>
       <x:c r="J143" s="0">
         <x:v>0</x:v>
@@ -6274,7 +6277,7 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B144" s="0" t="s">
-        <x:v>271</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="C144" s="0">
         <x:v>5000000</x:v>
@@ -6295,21 +6298,21 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I144" s="0">
-        <x:v>9.87</x:v>
+        <x:v>10.01</x:v>
       </x:c>
       <x:c r="J144" s="0">
         <x:v>7.82</x:v>
       </x:c>
       <x:c r="K144" s="0" t="s">
-        <x:v>272</x:v>
+        <x:v>273</x:v>
       </x:c>
     </x:row>
     <x:row r="145" spans="1:11">
       <x:c r="A145" s="0" t="s">
-        <x:v>273</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="B145" s="0" t="s">
-        <x:v>274</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="C145" s="0">
         <x:v>905991</x:v>
@@ -6330,7 +6333,7 @@
         <x:v>0.13</x:v>
       </x:c>
       <x:c r="I145" s="0">
-        <x:v>15.75</x:v>
+        <x:v>15.88</x:v>
       </x:c>
       <x:c r="J145" s="0">
         <x:v>19.26</x:v>
@@ -6341,10 +6344,10 @@
     </x:row>
     <x:row r="146" spans="1:11">
       <x:c r="A146" s="0" t="s">
-        <x:v>275</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="B146" s="0" t="s">
-        <x:v>276</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="C146" s="0" t="s">
         <x:v>13</x:v>
@@ -6365,7 +6368,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I146" s="0">
-        <x:v>41.36</x:v>
+        <x:v>42.26</x:v>
       </x:c>
       <x:c r="J146" s="0">
         <x:v>0</x:v>
@@ -6373,10 +6376,10 @@
     </x:row>
     <x:row r="147" spans="1:11">
       <x:c r="A147" s="0" t="s">
-        <x:v>255</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="B147" s="0" t="s">
-        <x:v>277</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="C147" s="0" t="s">
         <x:v>13</x:v>
@@ -6397,7 +6400,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I147" s="0">
-        <x:v>510</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="J147" s="0">
         <x:v>0</x:v>
@@ -6405,10 +6408,10 @@
     </x:row>
     <x:row r="148" spans="1:11">
       <x:c r="A148" s="0" t="s">
-        <x:v>278</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="B148" s="0" t="s">
-        <x:v>279</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="C148" s="0">
         <x:v>53584</x:v>
@@ -6429,21 +6432,21 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I148" s="0">
-        <x:v>260</x:v>
+        <x:v>255.25</x:v>
       </x:c>
       <x:c r="J148" s="0">
         <x:v>154.36</x:v>
       </x:c>
       <x:c r="K148" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="149" spans="1:11">
       <x:c r="A149" s="0" t="s">
-        <x:v>280</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="B149" s="0" t="s">
-        <x:v>281</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="C149" s="0">
         <x:v>7550000</x:v>
@@ -6464,21 +6467,21 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I149" s="0">
-        <x:v>14.99</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J149" s="0">
         <x:v>14.81</x:v>
       </x:c>
       <x:c r="K149" s="0" t="s">
-        <x:v>282</x:v>
+        <x:v>283</x:v>
       </x:c>
     </x:row>
     <x:row r="150" spans="1:11">
       <x:c r="A150" s="0" t="s">
-        <x:v>283</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="B150" s="0" t="s">
-        <x:v>284</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="C150" s="0">
         <x:v>2097716</x:v>
@@ -6499,21 +6502,21 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I150" s="0">
-        <x:v>1.26</x:v>
+        <x:v>1.24</x:v>
       </x:c>
       <x:c r="J150" s="0">
         <x:v>13.82</x:v>
       </x:c>
       <x:c r="K150" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="151" spans="1:11">
       <x:c r="A151" s="0" t="s">
-        <x:v>285</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="B151" s="0" t="s">
-        <x:v>286</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="C151" s="0">
         <x:v>5185302</x:v>
@@ -6534,21 +6537,21 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I151" s="0">
-        <x:v>5.81</x:v>
+        <x:v>5.77</x:v>
       </x:c>
       <x:c r="J151" s="0">
         <x:v>7.15</x:v>
       </x:c>
       <x:c r="K151" s="0" t="s">
-        <x:v>246</x:v>
+        <x:v>247</x:v>
       </x:c>
     </x:row>
     <x:row r="152" spans="1:11">
       <x:c r="A152" s="0" t="s">
-        <x:v>287</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B152" s="0" t="s">
-        <x:v>288</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="C152" s="0">
         <x:v>669111</x:v>
@@ -6569,21 +6572,21 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I152" s="0">
-        <x:v>751</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="J152" s="0">
         <x:v>226</x:v>
       </x:c>
       <x:c r="K152" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="153" spans="1:11">
       <x:c r="A153" s="0" t="s">
-        <x:v>255</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="B153" s="0" t="s">
-        <x:v>288</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="C153" s="0">
         <x:v>38840</x:v>
@@ -6604,21 +6607,21 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I153" s="0">
-        <x:v>510</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="J153" s="0">
         <x:v>242.84</x:v>
       </x:c>
       <x:c r="K153" s="0" t="s">
-        <x:v>284</x:v>
+        <x:v>285</x:v>
       </x:c>
     </x:row>
     <x:row r="154" spans="1:11">
       <x:c r="A154" s="0" t="s">
-        <x:v>280</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="B154" s="0" t="s">
-        <x:v>289</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C154" s="0">
         <x:v>2250000</x:v>
@@ -6639,21 +6642,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I154" s="0">
-        <x:v>14.99</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J154" s="0">
         <x:v>14.11</x:v>
       </x:c>
       <x:c r="K154" s="0" t="s">
-        <x:v>290</x:v>
+        <x:v>291</x:v>
       </x:c>
     </x:row>
     <x:row r="155" spans="1:11">
       <x:c r="A155" s="0" t="s">
-        <x:v>283</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="B155" s="0" t="s">
-        <x:v>291</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="C155" s="0">
         <x:v>1500000</x:v>
@@ -6674,21 +6677,21 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I155" s="0">
-        <x:v>1.26</x:v>
+        <x:v>1.24</x:v>
       </x:c>
       <x:c r="J155" s="0">
         <x:v>14.58</x:v>
       </x:c>
       <x:c r="K155" s="0" t="s">
-        <x:v>290</x:v>
+        <x:v>291</x:v>
       </x:c>
     </x:row>
     <x:row r="156" spans="1:11">
       <x:c r="A156" s="0" t="s">
-        <x:v>292</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="B156" s="0" t="s">
-        <x:v>293</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="C156" s="0">
         <x:v>1430040</x:v>
@@ -6709,7 +6712,7 @@
         <x:v>1.51</x:v>
       </x:c>
       <x:c r="I156" s="0">
-        <x:v>137.7</x:v>
+        <x:v>138.1</x:v>
       </x:c>
       <x:c r="J156" s="0">
         <x:v>138.67</x:v>
@@ -6720,10 +6723,10 @@
     </x:row>
     <x:row r="157" spans="1:11">
       <x:c r="A157" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B157" s="0" t="s">
-        <x:v>294</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="C157" s="0" t="s">
         <x:v>13</x:v>
@@ -6744,7 +6747,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I157" s="0">
-        <x:v>294.5</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="J157" s="0">
         <x:v>0</x:v>
@@ -6752,10 +6755,10 @@
     </x:row>
     <x:row r="158" spans="1:11">
       <x:c r="A158" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B158" s="0" t="s">
-        <x:v>295</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="C158" s="0">
         <x:v>845945</x:v>
@@ -6776,21 +6779,21 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I158" s="0">
-        <x:v>4.02</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="J158" s="0">
         <x:v>11.89</x:v>
       </x:c>
       <x:c r="K158" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
     </x:row>
     <x:row r="159" spans="1:11">
       <x:c r="A159" s="0" t="s">
-        <x:v>296</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="B159" s="0" t="s">
-        <x:v>297</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="C159" s="0">
         <x:v>21446</x:v>
@@ -6811,21 +6814,21 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I159" s="0">
-        <x:v>47.5</x:v>
+        <x:v>45.92</x:v>
       </x:c>
       <x:c r="J159" s="0">
         <x:v>94</x:v>
       </x:c>
       <x:c r="K159" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="160" spans="1:11">
       <x:c r="A160" s="0" t="s">
-        <x:v>298</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="B160" s="0" t="s">
-        <x:v>299</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C160" s="0">
         <x:v>850000</x:v>
@@ -6846,21 +6849,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I160" s="0">
-        <x:v>7.11</x:v>
+        <x:v>7.02</x:v>
       </x:c>
       <x:c r="J160" s="0">
         <x:v>7.7</x:v>
       </x:c>
       <x:c r="K160" s="0" t="s">
-        <x:v>229</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="161" spans="1:11">
       <x:c r="A161" s="0" t="s">
-        <x:v>300</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="B161" s="0" t="s">
-        <x:v>301</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="C161" s="0">
         <x:v>15000000</x:v>
@@ -6881,21 +6884,21 @@
         <x:v>0.22</x:v>
       </x:c>
       <x:c r="I161" s="0">
-        <x:v>3.11</x:v>
+        <x:v>3.21</x:v>
       </x:c>
       <x:c r="J161" s="0">
         <x:v>1.6</x:v>
       </x:c>
       <x:c r="K161" s="0" t="s">
-        <x:v>302</x:v>
+        <x:v>303</x:v>
       </x:c>
     </x:row>
     <x:row r="162" spans="1:11">
       <x:c r="A162" s="0" t="s">
-        <x:v>303</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="B162" s="0" t="s">
-        <x:v>304</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="C162" s="0">
         <x:v>6397124</x:v>
@@ -6916,21 +6919,21 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I162" s="0">
-        <x:v>4.11</x:v>
+        <x:v>4.14</x:v>
       </x:c>
       <x:c r="J162" s="0">
         <x:v>19.21</x:v>
       </x:c>
       <x:c r="K162" s="0" t="s">
-        <x:v>305</x:v>
+        <x:v>306</x:v>
       </x:c>
     </x:row>
     <x:row r="163" spans="1:11">
       <x:c r="A163" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B163" s="0" t="s">
-        <x:v>306</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="C163" s="0">
         <x:v>17495257</x:v>
@@ -6951,21 +6954,21 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I163" s="0">
-        <x:v>18.66</x:v>
+        <x:v>18.16</x:v>
       </x:c>
       <x:c r="J163" s="0">
         <x:v>23.4</x:v>
       </x:c>
       <x:c r="K163" s="0" t="s">
-        <x:v>307</x:v>
+        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="164" spans="1:11">
       <x:c r="A164" s="0" t="s">
-        <x:v>308</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="B164" s="0" t="s">
-        <x:v>309</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="C164" s="0">
         <x:v>9350000</x:v>
@@ -6986,21 +6989,21 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="I164" s="0">
-        <x:v>2.43</x:v>
+        <x:v>2.56</x:v>
       </x:c>
       <x:c r="J164" s="0">
         <x:v>7.44</x:v>
       </x:c>
       <x:c r="K164" s="0" t="s">
-        <x:v>310</x:v>
+        <x:v>311</x:v>
       </x:c>
     </x:row>
     <x:row r="165" spans="1:11">
       <x:c r="A165" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B165" s="0" t="s">
-        <x:v>311</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="C165" s="0">
         <x:v>1468255</x:v>
@@ -7021,21 +7024,21 @@
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="I165" s="0">
-        <x:v>23.34</x:v>
+        <x:v>23.4</x:v>
       </x:c>
       <x:c r="J165" s="0">
         <x:v>51.7</x:v>
       </x:c>
       <x:c r="K165" s="0" t="s">
-        <x:v>312</x:v>
+        <x:v>313</x:v>
       </x:c>
     </x:row>
     <x:row r="166" spans="1:11">
       <x:c r="A166" s="0" t="s">
-        <x:v>313</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="B166" s="0" t="s">
-        <x:v>314</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="C166" s="0">
         <x:v>500000</x:v>
@@ -7056,21 +7059,21 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I166" s="0">
-        <x:v>2.27</x:v>
+        <x:v>2.23</x:v>
       </x:c>
       <x:c r="J166" s="0">
         <x:v>26.8</x:v>
       </x:c>
       <x:c r="K166" s="0" t="s">
-        <x:v>188</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="167" spans="1:11">
       <x:c r="A167" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B167" s="0" t="s">
-        <x:v>315</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="C167" s="0">
         <x:v>725000</x:v>
@@ -7091,21 +7094,21 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="I167" s="0">
-        <x:v>40.2</x:v>
+        <x:v>39.94</x:v>
       </x:c>
       <x:c r="J167" s="0">
         <x:v>66.95</x:v>
       </x:c>
       <x:c r="K167" s="0" t="s">
-        <x:v>316</x:v>
+        <x:v>317</x:v>
       </x:c>
     </x:row>
     <x:row r="168" spans="1:11">
       <x:c r="A168" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B168" s="0" t="s">
-        <x:v>317</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="C168" s="0">
         <x:v>1060056</x:v>
@@ -7126,21 +7129,21 @@
         <x:v>0.44</x:v>
       </x:c>
       <x:c r="I168" s="0">
-        <x:v>221.8</x:v>
+        <x:v>220.9</x:v>
       </x:c>
       <x:c r="J168" s="0">
         <x:v>57.32</x:v>
       </x:c>
       <x:c r="K168" s="0" t="s">
-        <x:v>318</x:v>
+        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="169" spans="1:11">
       <x:c r="A169" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B169" s="0" t="s">
-        <x:v>319</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="C169" s="0">
         <x:v>132750000</x:v>
@@ -7161,21 +7164,21 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I169" s="0">
-        <x:v>2.76</x:v>
+        <x:v>2.73</x:v>
       </x:c>
       <x:c r="J169" s="0">
         <x:v>4.26</x:v>
       </x:c>
       <x:c r="K169" s="0" t="s">
-        <x:v>246</x:v>
+        <x:v>247</x:v>
       </x:c>
     </x:row>
     <x:row r="170" spans="1:11">
       <x:c r="A170" s="0" t="s">
-        <x:v>320</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="B170" s="0" t="s">
-        <x:v>321</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="C170" s="0">
         <x:v>373000</x:v>
@@ -7196,21 +7199,21 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I170" s="0">
-        <x:v>8.45</x:v>
+        <x:v>8.42</x:v>
       </x:c>
       <x:c r="J170" s="0">
         <x:v>63.77</x:v>
       </x:c>
       <x:c r="K170" s="0" t="s">
-        <x:v>322</x:v>
+        <x:v>323</x:v>
       </x:c>
     </x:row>
     <x:row r="171" spans="1:11">
       <x:c r="A171" s="0" t="s">
-        <x:v>323</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="B171" s="0" t="s">
-        <x:v>324</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="C171" s="0">
         <x:v>10000000</x:v>
@@ -7231,13 +7234,13 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I171" s="0">
-        <x:v>10.51</x:v>
+        <x:v>10.69</x:v>
       </x:c>
       <x:c r="J171" s="0">
         <x:v>13.33</x:v>
       </x:c>
       <x:c r="K171" s="0" t="s">
-        <x:v>325</x:v>
+        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="172" spans="1:11">
@@ -7245,7 +7248,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B172" s="0" t="s">
-        <x:v>326</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="C172" s="0">
         <x:v>66142950</x:v>
@@ -7266,21 +7269,21 @@
         <x:v>2.71</x:v>
       </x:c>
       <x:c r="I172" s="0">
-        <x:v>7.06</x:v>
+        <x:v>7.24</x:v>
       </x:c>
       <x:c r="J172" s="0">
         <x:v>5.82</x:v>
       </x:c>
       <x:c r="K172" s="0" t="s">
-        <x:v>327</x:v>
+        <x:v>328</x:v>
       </x:c>
     </x:row>
     <x:row r="173" spans="1:11">
       <x:c r="A173" s="0" t="s">
-        <x:v>328</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="B173" s="0" t="s">
-        <x:v>329</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="C173" s="0">
         <x:v>3081843</x:v>
@@ -7301,13 +7304,13 @@
         <x:v>0.66</x:v>
       </x:c>
       <x:c r="I173" s="0">
-        <x:v>5.87</x:v>
+        <x:v>5.77</x:v>
       </x:c>
       <x:c r="J173" s="0">
         <x:v>14.27</x:v>
       </x:c>
       <x:c r="K173" s="0" t="s">
-        <x:v>271</x:v>
+        <x:v>272</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Site guncellemesi - 10.09.2026 18:36
</commit_message>
<xml_diff>
--- a/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
+++ b/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
@@ -217,7 +217,7 @@
     <x:t>12.06.2026</x:t>
   </x:si>
   <x:si>
-    <x:t>08.09.2026</x:t>
+    <x:t>10.09.2026</x:t>
   </x:si>
   <x:si>
     <x:t>KLSYN</x:t>
@@ -1421,7 +1421,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>8.94</x:v>
+        <x:v>8.68</x:v>
       </x:c>
       <x:c r="J2" s="0">
         <x:v>0</x:v>
@@ -1453,7 +1453,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>4.72</x:v>
+        <x:v>5.15</x:v>
       </x:c>
       <x:c r="J3" s="0">
         <x:v>0</x:v>
@@ -1485,7 +1485,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>6.65</x:v>
+        <x:v>6.66</x:v>
       </x:c>
       <x:c r="J4" s="0">
         <x:v>0</x:v>
@@ -1517,7 +1517,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>9.23</x:v>
+        <x:v>9.2</x:v>
       </x:c>
       <x:c r="J5" s="0">
         <x:v>8.74</x:v>
@@ -1552,7 +1552,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>27.46</x:v>
+        <x:v>26.1</x:v>
       </x:c>
       <x:c r="J6" s="0">
         <x:v>0</x:v>
@@ -1584,7 +1584,7 @@
         <x:v>3.7</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>6.63</x:v>
+        <x:v>6.67</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>6.99</x:v>
@@ -1619,7 +1619,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>21.18</x:v>
+        <x:v>21.22</x:v>
       </x:c>
       <x:c r="J8" s="0">
         <x:v>23.68</x:v>
@@ -1654,7 +1654,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>7.24</x:v>
+        <x:v>7.12</x:v>
       </x:c>
       <x:c r="J9" s="0">
         <x:v>8.39</x:v>
@@ -1689,7 +1689,7 @@
         <x:v>3.83</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>13.74</x:v>
+        <x:v>13.75</x:v>
       </x:c>
       <x:c r="J10" s="0">
         <x:v>0.76</x:v>
@@ -1724,7 +1724,7 @@
         <x:v>7.98</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>4.69</x:v>
+        <x:v>4.76</x:v>
       </x:c>
       <x:c r="J11" s="0">
         <x:v>1.47</x:v>
@@ -1759,7 +1759,7 @@
         <x:v>8.08</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>15</x:v>
+        <x:v>14.5</x:v>
       </x:c>
       <x:c r="J12" s="0">
         <x:v>0.73</x:v>
@@ -1794,7 +1794,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>65</x:v>
+        <x:v>66.5</x:v>
       </x:c>
       <x:c r="J13" s="0">
         <x:v>64.98</x:v>
@@ -1829,7 +1829,7 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>1.33</x:v>
+        <x:v>1.35</x:v>
       </x:c>
       <x:c r="J14" s="0">
         <x:v>1.33</x:v>
@@ -1864,7 +1864,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>136.4</x:v>
+        <x:v>136.1</x:v>
       </x:c>
       <x:c r="J15" s="0">
         <x:v>0</x:v>
@@ -1896,7 +1896,7 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>5.54</x:v>
+        <x:v>5.44</x:v>
       </x:c>
       <x:c r="J16" s="0">
         <x:v>6.13</x:v>
@@ -1931,7 +1931,7 @@
         <x:v>0.43</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>10.01</x:v>
+        <x:v>9.93</x:v>
       </x:c>
       <x:c r="J17" s="0">
         <x:v>9.9</x:v>
@@ -1966,7 +1966,7 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>9.23</x:v>
+        <x:v>9.2</x:v>
       </x:c>
       <x:c r="J18" s="0">
         <x:v>9.69</x:v>
@@ -2001,7 +2001,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>18.8</x:v>
+        <x:v>18.44</x:v>
       </x:c>
       <x:c r="J19" s="0">
         <x:v>0</x:v>
@@ -2033,7 +2033,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>1.7</x:v>
+        <x:v>1.67</x:v>
       </x:c>
       <x:c r="J20" s="0">
         <x:v>0</x:v>
@@ -2065,7 +2065,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>16.52</x:v>
+        <x:v>16.12</x:v>
       </x:c>
       <x:c r="J21" s="0">
         <x:v>15.87</x:v>
@@ -2100,7 +2100,7 @@
         <x:v>0.55</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>17.61</x:v>
+        <x:v>17.85</x:v>
       </x:c>
       <x:c r="J22" s="0">
         <x:v>19.08</x:v>
@@ -2135,7 +2135,7 @@
         <x:v>0.65</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>3.86</x:v>
+        <x:v>4.01</x:v>
       </x:c>
       <x:c r="J23" s="0">
         <x:v>3.49</x:v>
@@ -2170,7 +2170,7 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>427.5</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="J24" s="0">
         <x:v>380.17</x:v>
@@ -2205,7 +2205,7 @@
         <x:v>1.29</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>69.5</x:v>
+        <x:v>70.65</x:v>
       </x:c>
       <x:c r="J25" s="0">
         <x:v>69.8</x:v>
@@ -2240,7 +2240,7 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>39.6</x:v>
+        <x:v>38.62</x:v>
       </x:c>
       <x:c r="J26" s="0">
         <x:v>38.82</x:v>
@@ -2275,7 +2275,7 @@
         <x:v>1.8</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>53.9</x:v>
+        <x:v>52.45</x:v>
       </x:c>
       <x:c r="J27" s="0">
         <x:v>48.23</x:v>
@@ -2292,7 +2292,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="C28" s="0">
-        <x:v>45660619</x:v>
+        <x:v>48947313</x:v>
       </x:c>
       <x:c r="D28" s="0">
         <x:v>25000000</x:v>
@@ -2301,19 +2301,19 @@
         <x:v>1000000000</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>1553431530</x:v>
+        <x:v>1674316254</x:v>
       </x:c>
       <x:c r="G28" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.55</x:v>
+        <x:v>1.66</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>37.2</x:v>
+        <x:v>37.24</x:v>
       </x:c>
       <x:c r="J28" s="0">
-        <x:v>34.02</x:v>
+        <x:v>34.21</x:v>
       </x:c>
       <x:c r="K28" s="0" t="s">
         <x:v>67</x:v>
@@ -2345,7 +2345,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>16.43</x:v>
+        <x:v>16.32</x:v>
       </x:c>
       <x:c r="J29" s="0">
         <x:v>5.49</x:v>
@@ -2380,7 +2380,7 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>24.86</x:v>
+        <x:v>23.62</x:v>
       </x:c>
       <x:c r="J30" s="0">
         <x:v>21.09</x:v>
@@ -2415,7 +2415,7 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>10.28</x:v>
+        <x:v>10.11</x:v>
       </x:c>
       <x:c r="J31" s="0">
         <x:v>10.31</x:v>
@@ -2482,7 +2482,7 @@
         <x:v>0.35</x:v>
       </x:c>
       <x:c r="I33" s="0">
-        <x:v>8.53</x:v>
+        <x:v>8.4</x:v>
       </x:c>
       <x:c r="J33" s="0">
         <x:v>7.46</x:v>
@@ -2517,7 +2517,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I34" s="0">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="J34" s="0">
         <x:v>0</x:v>
@@ -2549,7 +2549,7 @@
         <x:v>0.82</x:v>
       </x:c>
       <x:c r="I35" s="0">
-        <x:v>18.59</x:v>
+        <x:v>18.8</x:v>
       </x:c>
       <x:c r="J35" s="0">
         <x:v>7.13</x:v>
@@ -2584,7 +2584,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I36" s="0">
-        <x:v>22.92</x:v>
+        <x:v>23.14</x:v>
       </x:c>
       <x:c r="J36" s="0">
         <x:v>28.89</x:v>
@@ -2619,7 +2619,7 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I37" s="0">
-        <x:v>9.43</x:v>
+        <x:v>9.52</x:v>
       </x:c>
       <x:c r="J37" s="0">
         <x:v>15.08</x:v>
@@ -2654,7 +2654,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I38" s="0">
-        <x:v>4.68</x:v>
+        <x:v>4.55</x:v>
       </x:c>
       <x:c r="J38" s="0">
         <x:v>0</x:v>
@@ -2686,7 +2686,7 @@
         <x:v>2.78</x:v>
       </x:c>
       <x:c r="I39" s="0">
-        <x:v>21.82</x:v>
+        <x:v>21.26</x:v>
       </x:c>
       <x:c r="J39" s="0">
         <x:v>23.25</x:v>
@@ -2703,7 +2703,7 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="C40" s="0">
-        <x:v>28532493</x:v>
+        <x:v>28921768</x:v>
       </x:c>
       <x:c r="D40" s="0">
         <x:v>80000000</x:v>
@@ -2712,22 +2712,22 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F40" s="0">
-        <x:v>794742815</x:v>
+        <x:v>809671512</x:v>
       </x:c>
       <x:c r="G40" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H40" s="0">
-        <x:v>1.1</x:v>
+        <x:v>1.11</x:v>
       </x:c>
       <x:c r="I40" s="0">
-        <x:v>38.42</x:v>
+        <x:v>39.24</x:v>
       </x:c>
       <x:c r="J40" s="0">
-        <x:v>27.85</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="K40" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:11">
@@ -2756,7 +2756,7 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I41" s="0">
-        <x:v>11.29</x:v>
+        <x:v>11.27</x:v>
       </x:c>
       <x:c r="J41" s="0">
         <x:v>13.34</x:v>
@@ -2791,7 +2791,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I42" s="0">
-        <x:v>37.26</x:v>
+        <x:v>38.08</x:v>
       </x:c>
       <x:c r="J42" s="0">
         <x:v>39.18</x:v>
@@ -2826,7 +2826,7 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="I43" s="0">
-        <x:v>61.45</x:v>
+        <x:v>63.75</x:v>
       </x:c>
       <x:c r="J43" s="0">
         <x:v>59.93</x:v>
@@ -2861,7 +2861,7 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="I44" s="0">
-        <x:v>5.69</x:v>
+        <x:v>5.65</x:v>
       </x:c>
       <x:c r="J44" s="0">
         <x:v>48.39</x:v>
@@ -2896,7 +2896,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I45" s="0">
-        <x:v>3.93</x:v>
+        <x:v>3.92</x:v>
       </x:c>
       <x:c r="J45" s="0">
         <x:v>0</x:v>
@@ -2928,7 +2928,7 @@
         <x:v>0.43</x:v>
       </x:c>
       <x:c r="I46" s="0">
-        <x:v>23.5</x:v>
+        <x:v>22.44</x:v>
       </x:c>
       <x:c r="J46" s="0">
         <x:v>45.09</x:v>
@@ -2945,7 +2945,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="C47" s="0">
-        <x:v>16715421</x:v>
+        <x:v>17473248</x:v>
       </x:c>
       <x:c r="D47" s="0">
         <x:v>35000000</x:v>
@@ -2954,22 +2954,22 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F47" s="0">
-        <x:v>145342995</x:v>
+        <x:v>152638225</x:v>
       </x:c>
       <x:c r="G47" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H47" s="0">
-        <x:v>4.18</x:v>
+        <x:v>4.37</x:v>
       </x:c>
       <x:c r="I47" s="0">
-        <x:v>9.42</x:v>
+        <x:v>9.4</x:v>
       </x:c>
       <x:c r="J47" s="0">
-        <x:v>8.7</x:v>
+        <x:v>8.74</x:v>
       </x:c>
       <x:c r="K47" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:11">
@@ -2998,7 +2998,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I48" s="0">
-        <x:v>77.8</x:v>
+        <x:v>73.5</x:v>
       </x:c>
       <x:c r="J48" s="0">
         <x:v>61.87</x:v>
@@ -3033,7 +3033,7 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I49" s="0">
-        <x:v>18.16</x:v>
+        <x:v>17.87</x:v>
       </x:c>
       <x:c r="J49" s="0">
         <x:v>21.06</x:v>
@@ -3068,7 +3068,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I50" s="0">
-        <x:v>5.69</x:v>
+        <x:v>5.65</x:v>
       </x:c>
       <x:c r="J50" s="0">
         <x:v>0</x:v>
@@ -3082,7 +3082,7 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="C51" s="0">
-        <x:v>103967273</x:v>
+        <x:v>104378690</x:v>
       </x:c>
       <x:c r="D51" s="0">
         <x:v>200000000</x:v>
@@ -3091,7 +3091,7 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F51" s="0">
-        <x:v>1016303268</x:v>
+        <x:v>1020837906</x:v>
       </x:c>
       <x:c r="G51" s="0">
         <x:v>0</x:v>
@@ -3100,13 +3100,13 @@
         <x:v>1.16</x:v>
       </x:c>
       <x:c r="I51" s="0">
-        <x:v>11.09</x:v>
+        <x:v>11.47</x:v>
       </x:c>
       <x:c r="J51" s="0">
         <x:v>9.78</x:v>
       </x:c>
       <x:c r="K51" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:11">
@@ -3135,7 +3135,7 @@
         <x:v>3.29</x:v>
       </x:c>
       <x:c r="I52" s="0">
-        <x:v>43.5</x:v>
+        <x:v>43.06</x:v>
       </x:c>
       <x:c r="J52" s="0">
         <x:v>23.95</x:v>
@@ -3170,7 +3170,7 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I53" s="0">
-        <x:v>427.5</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="J53" s="0">
         <x:v>528.86</x:v>
@@ -3205,7 +3205,7 @@
         <x:v>0.94</x:v>
       </x:c>
       <x:c r="I54" s="0">
-        <x:v>38.42</x:v>
+        <x:v>39.24</x:v>
       </x:c>
       <x:c r="J54" s="0">
         <x:v>24.19</x:v>
@@ -3240,7 +3240,7 @@
         <x:v>0.52</x:v>
       </x:c>
       <x:c r="I55" s="0">
-        <x:v>11.09</x:v>
+        <x:v>11.47</x:v>
       </x:c>
       <x:c r="J55" s="0">
         <x:v>10.74</x:v>
@@ -3275,7 +3275,7 @@
         <x:v>0.69</x:v>
       </x:c>
       <x:c r="I56" s="0">
-        <x:v>6.65</x:v>
+        <x:v>6.66</x:v>
       </x:c>
       <x:c r="J56" s="0">
         <x:v>6.01</x:v>
@@ -3310,7 +3310,7 @@
         <x:v>1.36</x:v>
       </x:c>
       <x:c r="I57" s="0">
-        <x:v>19</x:v>
+        <x:v>18.6</x:v>
       </x:c>
       <x:c r="J57" s="0">
         <x:v>25.45</x:v>
@@ -3345,7 +3345,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I58" s="0">
-        <x:v>3.74</x:v>
+        <x:v>4.06</x:v>
       </x:c>
       <x:c r="J58" s="0">
         <x:v>4.46</x:v>
@@ -3380,7 +3380,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I59" s="0">
-        <x:v>6.63</x:v>
+        <x:v>6.67</x:v>
       </x:c>
       <x:c r="J59" s="0">
         <x:v>12.82</x:v>
@@ -3415,7 +3415,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I60" s="0">
-        <x:v>33.1</x:v>
+        <x:v>31.02</x:v>
       </x:c>
       <x:c r="J60" s="0">
         <x:v>0</x:v>
@@ -3447,7 +3447,7 @@
         <x:v>0.83</x:v>
       </x:c>
       <x:c r="I61" s="0">
-        <x:v>3.03</x:v>
+        <x:v>2.98</x:v>
       </x:c>
       <x:c r="J61" s="0">
         <x:v>52.14</x:v>
@@ -3482,7 +3482,7 @@
         <x:v>1.83</x:v>
       </x:c>
       <x:c r="I62" s="0">
-        <x:v>36.7</x:v>
+        <x:v>36.8</x:v>
       </x:c>
       <x:c r="J62" s="0">
         <x:v>39.62</x:v>
@@ -3499,7 +3499,7 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="C63" s="0">
-        <x:v>3729828</x:v>
+        <x:v>3799828</x:v>
       </x:c>
       <x:c r="D63" s="0">
         <x:v>3000000</x:v>
@@ -3508,22 +3508,22 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F63" s="0">
-        <x:v>176220944</x:v>
+        <x:v>177844244</x:v>
       </x:c>
       <x:c r="G63" s="0">
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="H63" s="0">
-        <x:v>0.93</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="I63" s="0">
-        <x:v>23.4</x:v>
+        <x:v>23.38</x:v>
       </x:c>
       <x:c r="J63" s="0">
-        <x:v>47.25</x:v>
+        <x:v>46.8</x:v>
       </x:c>
       <x:c r="K63" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:11">
@@ -3552,7 +3552,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I64" s="0">
-        <x:v>26.02</x:v>
+        <x:v>25.84</x:v>
       </x:c>
       <x:c r="J64" s="0">
         <x:v>0</x:v>
@@ -3584,7 +3584,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I65" s="0">
-        <x:v>3.9</x:v>
+        <x:v>3.89</x:v>
       </x:c>
       <x:c r="J65" s="0">
         <x:v>4.47</x:v>
@@ -3619,7 +3619,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I66" s="0">
-        <x:v>39.94</x:v>
+        <x:v>39.3</x:v>
       </x:c>
       <x:c r="J66" s="0">
         <x:v>0</x:v>
@@ -3651,7 +3651,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I67" s="0">
-        <x:v>301</x:v>
+        <x:v>299.25</x:v>
       </x:c>
       <x:c r="J67" s="0">
         <x:v>299.91</x:v>
@@ -3686,7 +3686,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I68" s="0">
-        <x:v>22.48</x:v>
+        <x:v>20.8</x:v>
       </x:c>
       <x:c r="J68" s="0">
         <x:v>0</x:v>
@@ -3718,7 +3718,7 @@
         <x:v>0.54</x:v>
       </x:c>
       <x:c r="I69" s="0">
-        <x:v>288</x:v>
+        <x:v>287.5</x:v>
       </x:c>
       <x:c r="J69" s="0">
         <x:v>83</x:v>
@@ -3753,7 +3753,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I70" s="0">
-        <x:v>35.18</x:v>
+        <x:v>34.58</x:v>
       </x:c>
       <x:c r="J70" s="0">
         <x:v>40.97</x:v>
@@ -3788,7 +3788,7 @@
         <x:v>0.62</x:v>
       </x:c>
       <x:c r="I71" s="0">
-        <x:v>21.18</x:v>
+        <x:v>21.22</x:v>
       </x:c>
       <x:c r="J71" s="0">
         <x:v>23.68</x:v>
@@ -3823,7 +3823,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I72" s="0">
-        <x:v>16.43</x:v>
+        <x:v>16.32</x:v>
       </x:c>
       <x:c r="J72" s="0">
         <x:v>5.49</x:v>
@@ -3858,7 +3858,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I73" s="0">
-        <x:v>16.52</x:v>
+        <x:v>16.12</x:v>
       </x:c>
       <x:c r="J73" s="0">
         <x:v>0</x:v>
@@ -3890,7 +3890,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I74" s="0">
-        <x:v>5.38</x:v>
+        <x:v>5.42</x:v>
       </x:c>
       <x:c r="J74" s="0">
         <x:v>0</x:v>
@@ -3922,7 +3922,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I75" s="0">
-        <x:v>6.66</x:v>
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="J75" s="0">
         <x:v>6.6</x:v>
@@ -3957,7 +3957,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I76" s="0">
-        <x:v>2.73</x:v>
+        <x:v>2.77</x:v>
       </x:c>
       <x:c r="J76" s="0">
         <x:v>3.98</x:v>
@@ -3992,7 +3992,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I77" s="0">
-        <x:v>19</x:v>
+        <x:v>18.6</x:v>
       </x:c>
       <x:c r="J77" s="0">
         <x:v>17.83</x:v>
@@ -4027,7 +4027,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I78" s="0">
-        <x:v>29.5</x:v>
+        <x:v>29.74</x:v>
       </x:c>
       <x:c r="J78" s="0">
         <x:v>38.06</x:v>
@@ -4062,7 +4062,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I79" s="0">
-        <x:v>220.9</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="J79" s="0">
         <x:v>0</x:v>
@@ -4094,7 +4094,7 @@
         <x:v>0.86</x:v>
       </x:c>
       <x:c r="I80" s="0">
-        <x:v>34.3</x:v>
+        <x:v>33.84</x:v>
       </x:c>
       <x:c r="J80" s="0">
         <x:v>41.13</x:v>
@@ -4129,7 +4129,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I81" s="0">
-        <x:v>4.63</x:v>
+        <x:v>4.58</x:v>
       </x:c>
       <x:c r="J81" s="0">
         <x:v>20.11</x:v>
@@ -4164,7 +4164,7 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I82" s="0">
-        <x:v>47</x:v>
+        <x:v>46.9</x:v>
       </x:c>
       <x:c r="J82" s="0">
         <x:v>39.43</x:v>
@@ -4199,7 +4199,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I83" s="0">
-        <x:v>18.58</x:v>
+        <x:v>19.06</x:v>
       </x:c>
       <x:c r="J83" s="0">
         <x:v>0</x:v>
@@ -4231,7 +4231,7 @@
         <x:v>0.12</x:v>
       </x:c>
       <x:c r="I84" s="0">
-        <x:v>21.5</x:v>
+        <x:v>21.64</x:v>
       </x:c>
       <x:c r="J84" s="0">
         <x:v>16.34</x:v>
@@ -4266,7 +4266,7 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="I85" s="0">
-        <x:v>72.6</x:v>
+        <x:v>72.3</x:v>
       </x:c>
       <x:c r="J85" s="0">
         <x:v>38.88</x:v>
@@ -4301,7 +4301,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I86" s="0">
-        <x:v>51.3</x:v>
+        <x:v>54.1</x:v>
       </x:c>
       <x:c r="J86" s="0">
         <x:v>0</x:v>
@@ -4333,7 +4333,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I87" s="0">
-        <x:v>12.34</x:v>
+        <x:v>11.94</x:v>
       </x:c>
       <x:c r="J87" s="0">
         <x:v>10.75</x:v>
@@ -4368,7 +4368,7 @@
         <x:v>2.16</x:v>
       </x:c>
       <x:c r="I88" s="0">
-        <x:v>34.3</x:v>
+        <x:v>34.26</x:v>
       </x:c>
       <x:c r="J88" s="0">
         <x:v>37.66</x:v>
@@ -4403,7 +4403,7 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I89" s="0">
-        <x:v>12.34</x:v>
+        <x:v>11.94</x:v>
       </x:c>
       <x:c r="J89" s="0">
         <x:v>161.23</x:v>
@@ -4438,7 +4438,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="I90" s="0">
-        <x:v>9.23</x:v>
+        <x:v>9.2</x:v>
       </x:c>
       <x:c r="J90" s="0">
         <x:v>15.68</x:v>
@@ -4473,7 +4473,7 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I91" s="0">
-        <x:v>1.97</x:v>
+        <x:v>1.95</x:v>
       </x:c>
       <x:c r="J91" s="0">
         <x:v>8.95</x:v>
@@ -4508,7 +4508,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I92" s="0">
-        <x:v>3.99</x:v>
+        <x:v>3.94</x:v>
       </x:c>
       <x:c r="J92" s="0">
         <x:v>0</x:v>
@@ -4540,7 +4540,7 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="I93" s="0">
-        <x:v>2.08</x:v>
+        <x:v>2.05</x:v>
       </x:c>
       <x:c r="J93" s="0">
         <x:v>4.93</x:v>
@@ -4575,7 +4575,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I94" s="0">
-        <x:v>101.8</x:v>
+        <x:v>101.6</x:v>
       </x:c>
       <x:c r="J94" s="0">
         <x:v>95.58</x:v>
@@ -4610,7 +4610,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I95" s="0">
-        <x:v>50.2</x:v>
+        <x:v>50.05</x:v>
       </x:c>
       <x:c r="J95" s="0">
         <x:v>0</x:v>
@@ -4642,7 +4642,7 @@
         <x:v>1.31</x:v>
       </x:c>
       <x:c r="I96" s="0">
-        <x:v>2.61</x:v>
+        <x:v>2.87</x:v>
       </x:c>
       <x:c r="J96" s="0">
         <x:v>2.45</x:v>
@@ -4677,7 +4677,7 @@
         <x:v>1.08</x:v>
       </x:c>
       <x:c r="I97" s="0">
-        <x:v>65</x:v>
+        <x:v>66.5</x:v>
       </x:c>
       <x:c r="J97" s="0">
         <x:v>58.33</x:v>
@@ -4712,7 +4712,7 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I98" s="0">
-        <x:v>24.86</x:v>
+        <x:v>23.62</x:v>
       </x:c>
       <x:c r="J98" s="0">
         <x:v>21.09</x:v>
@@ -4747,7 +4747,7 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I99" s="0">
-        <x:v>26.5</x:v>
+        <x:v>27.88</x:v>
       </x:c>
       <x:c r="J99" s="0">
         <x:v>16.87</x:v>
@@ -4782,7 +4782,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I100" s="0">
-        <x:v>5.54</x:v>
+        <x:v>5.44</x:v>
       </x:c>
       <x:c r="J100" s="0">
         <x:v>11.99</x:v>
@@ -4817,7 +4817,7 @@
         <x:v>0.16</x:v>
       </x:c>
       <x:c r="I101" s="0">
-        <x:v>17.27</x:v>
+        <x:v>17.53</x:v>
       </x:c>
       <x:c r="J101" s="0">
         <x:v>22.05</x:v>
@@ -4852,7 +4852,7 @@
         <x:v>1.45</x:v>
       </x:c>
       <x:c r="I102" s="0">
-        <x:v>86.05</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="J102" s="0">
         <x:v>68.15</x:v>
@@ -4887,7 +4887,7 @@
         <x:v>0.68</x:v>
       </x:c>
       <x:c r="I103" s="0">
-        <x:v>30.8</x:v>
+        <x:v>30.5</x:v>
       </x:c>
       <x:c r="J103" s="0">
         <x:v>35.38</x:v>
@@ -4922,7 +4922,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I104" s="0">
-        <x:v>6.9</x:v>
+        <x:v>6.83</x:v>
       </x:c>
       <x:c r="J104" s="0">
         <x:v>0</x:v>
@@ -4954,7 +4954,7 @@
         <x:v>0.27</x:v>
       </x:c>
       <x:c r="I105" s="0">
-        <x:v>9</x:v>
+        <x:v>8.94</x:v>
       </x:c>
       <x:c r="J105" s="0">
         <x:v>19.79</x:v>
@@ -4989,7 +4989,7 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I106" s="0">
-        <x:v>10.77</x:v>
+        <x:v>10.79</x:v>
       </x:c>
       <x:c r="J106" s="0">
         <x:v>13.15</x:v>
@@ -5024,7 +5024,7 @@
         <x:v>0.92</x:v>
       </x:c>
       <x:c r="I107" s="0">
-        <x:v>11.37</x:v>
+        <x:v>11.29</x:v>
       </x:c>
       <x:c r="J107" s="0">
         <x:v>10.98</x:v>
@@ -5059,7 +5059,7 @@
         <x:v>3.45</x:v>
       </x:c>
       <x:c r="I108" s="0">
-        <x:v>1.7</x:v>
+        <x:v>1.67</x:v>
       </x:c>
       <x:c r="J108" s="0">
         <x:v>4.03</x:v>
@@ -5094,7 +5094,7 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="I109" s="0">
-        <x:v>199.5</x:v>
+        <x:v>219.4</x:v>
       </x:c>
       <x:c r="J109" s="0">
         <x:v>284.58</x:v>
@@ -5129,7 +5129,7 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="I110" s="0">
-        <x:v>5.88</x:v>
+        <x:v>6.46</x:v>
       </x:c>
       <x:c r="J110" s="0">
         <x:v>38.02</x:v>
@@ -5164,7 +5164,7 @@
         <x:v>1.67</x:v>
       </x:c>
       <x:c r="I111" s="0">
-        <x:v>195.6</x:v>
+        <x:v>195.8</x:v>
       </x:c>
       <x:c r="J111" s="0">
         <x:v>83.62</x:v>
@@ -5199,7 +5199,7 @@
         <x:v>4.31</x:v>
       </x:c>
       <x:c r="I112" s="0">
-        <x:v>30.7</x:v>
+        <x:v>30.62</x:v>
       </x:c>
       <x:c r="J112" s="0">
         <x:v>17.65</x:v>
@@ -5234,7 +5234,7 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I113" s="0">
-        <x:v>8.94</x:v>
+        <x:v>8.68</x:v>
       </x:c>
       <x:c r="J113" s="0">
         <x:v>15.92</x:v>
@@ -5269,7 +5269,7 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I114" s="0">
-        <x:v>5.31</x:v>
+        <x:v>5.38</x:v>
       </x:c>
       <x:c r="J114" s="0">
         <x:v>40.97</x:v>
@@ -5304,7 +5304,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I115" s="0">
-        <x:v>10.17</x:v>
+        <x:v>11.18</x:v>
       </x:c>
       <x:c r="J115" s="0">
         <x:v>0</x:v>
@@ -5336,7 +5336,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I116" s="0">
-        <x:v>15.02</x:v>
+        <x:v>14.64</x:v>
       </x:c>
       <x:c r="J116" s="0">
         <x:v>16.42</x:v>
@@ -5371,7 +5371,7 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I117" s="0">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="J117" s="0">
         <x:v>31.92</x:v>
@@ -5406,7 +5406,7 @@
         <x:v>3.13</x:v>
       </x:c>
       <x:c r="I118" s="0">
-        <x:v>116.3</x:v>
+        <x:v>116.6</x:v>
       </x:c>
       <x:c r="J118" s="0">
         <x:v>94.36</x:v>
@@ -5441,7 +5441,7 @@
         <x:v>3.66</x:v>
       </x:c>
       <x:c r="I119" s="0">
-        <x:v>4.69</x:v>
+        <x:v>4.68</x:v>
       </x:c>
       <x:c r="J119" s="0">
         <x:v>4.76</x:v>
@@ -5476,7 +5476,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I120" s="0">
-        <x:v>427.5</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="J120" s="0">
         <x:v>429.82</x:v>
@@ -5511,7 +5511,7 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I121" s="0">
-        <x:v>3.06</x:v>
+        <x:v>3.05</x:v>
       </x:c>
       <x:c r="J121" s="0">
         <x:v>2.64</x:v>
@@ -5546,7 +5546,7 @@
         <x:v>1.45</x:v>
       </x:c>
       <x:c r="I122" s="0">
-        <x:v>13.23</x:v>
+        <x:v>13.16</x:v>
       </x:c>
       <x:c r="J122" s="0">
         <x:v>8.23</x:v>
@@ -5581,7 +5581,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I123" s="0">
-        <x:v>2.84</x:v>
+        <x:v>2.81</x:v>
       </x:c>
       <x:c r="J123" s="0">
         <x:v>0</x:v>
@@ -5613,7 +5613,7 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I124" s="0">
-        <x:v>27.6</x:v>
+        <x:v>27.36</x:v>
       </x:c>
       <x:c r="J124" s="0">
         <x:v>23.83</x:v>
@@ -5683,7 +5683,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I126" s="0">
-        <x:v>2.63</x:v>
+        <x:v>2.71</x:v>
       </x:c>
       <x:c r="J126" s="0">
         <x:v>0</x:v>
@@ -5715,7 +5715,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I127" s="0">
-        <x:v>38.42</x:v>
+        <x:v>39.24</x:v>
       </x:c>
       <x:c r="J127" s="0">
         <x:v>20.53</x:v>
@@ -5750,7 +5750,7 @@
         <x:v>1.24</x:v>
       </x:c>
       <x:c r="I128" s="0">
-        <x:v>11.09</x:v>
+        <x:v>11.47</x:v>
       </x:c>
       <x:c r="J128" s="0">
         <x:v>4.48</x:v>
@@ -5785,7 +5785,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I129" s="0">
-        <x:v>3.71</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="J129" s="0">
         <x:v>0</x:v>
@@ -5817,7 +5817,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I130" s="0">
-        <x:v>7.09</x:v>
+        <x:v>7.08</x:v>
       </x:c>
       <x:c r="J130" s="0">
         <x:v>0</x:v>
@@ -5849,7 +5849,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I131" s="0">
-        <x:v>154.2</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="J131" s="0">
         <x:v>50.97</x:v>
@@ -5884,7 +5884,7 @@
         <x:v>5.91</x:v>
       </x:c>
       <x:c r="I132" s="0">
-        <x:v>16.52</x:v>
+        <x:v>16.12</x:v>
       </x:c>
       <x:c r="J132" s="0">
         <x:v>10.93</x:v>
@@ -5919,7 +5919,7 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="I133" s="0">
-        <x:v>38.2</x:v>
+        <x:v>36.5</x:v>
       </x:c>
       <x:c r="J133" s="0">
         <x:v>38.14</x:v>
@@ -5954,7 +5954,7 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I134" s="0">
-        <x:v>139.5</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="J134" s="0">
         <x:v>39.56</x:v>
@@ -5989,7 +5989,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I135" s="0">
-        <x:v>545</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="J135" s="0">
         <x:v>0</x:v>
@@ -6056,7 +6056,7 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I137" s="0">
-        <x:v>35.52</x:v>
+        <x:v>34.62</x:v>
       </x:c>
       <x:c r="J137" s="0">
         <x:v>25.74</x:v>
@@ -6091,7 +6091,7 @@
         <x:v>1.9</x:v>
       </x:c>
       <x:c r="I138" s="0">
-        <x:v>17.17</x:v>
+        <x:v>17.19</x:v>
       </x:c>
       <x:c r="J138" s="0">
         <x:v>15.2</x:v>
@@ -6126,7 +6126,7 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="I139" s="0">
-        <x:v>26.22</x:v>
+        <x:v>24.66</x:v>
       </x:c>
       <x:c r="J139" s="0">
         <x:v>15.05</x:v>
@@ -6161,7 +6161,7 @@
         <x:v>5.09</x:v>
       </x:c>
       <x:c r="I140" s="0">
-        <x:v>13</x:v>
+        <x:v>12.72</x:v>
       </x:c>
       <x:c r="J140" s="0">
         <x:v>16.65</x:v>
@@ -6196,7 +6196,7 @@
         <x:v>1.89</x:v>
       </x:c>
       <x:c r="I141" s="0">
-        <x:v>16.63</x:v>
+        <x:v>16.71</x:v>
       </x:c>
       <x:c r="J141" s="0">
         <x:v>11.29</x:v>
@@ -6231,7 +6231,7 @@
         <x:v>0.93</x:v>
       </x:c>
       <x:c r="I142" s="0">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="J142" s="0">
         <x:v>30.45</x:v>
@@ -6266,7 +6266,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I143" s="0">
-        <x:v>2.09</x:v>
+        <x:v>2.05</x:v>
       </x:c>
       <x:c r="J143" s="0">
         <x:v>0</x:v>
@@ -6298,7 +6298,7 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I144" s="0">
-        <x:v>10.01</x:v>
+        <x:v>9.93</x:v>
       </x:c>
       <x:c r="J144" s="0">
         <x:v>7.82</x:v>
@@ -6333,7 +6333,7 @@
         <x:v>0.13</x:v>
       </x:c>
       <x:c r="I145" s="0">
-        <x:v>15.88</x:v>
+        <x:v>17.46</x:v>
       </x:c>
       <x:c r="J145" s="0">
         <x:v>19.26</x:v>
@@ -6368,7 +6368,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I146" s="0">
-        <x:v>42.26</x:v>
+        <x:v>41.22</x:v>
       </x:c>
       <x:c r="J146" s="0">
         <x:v>0</x:v>
@@ -6400,7 +6400,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I147" s="0">
-        <x:v>545</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="J147" s="0">
         <x:v>0</x:v>
@@ -6432,7 +6432,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I148" s="0">
-        <x:v>255.25</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="J148" s="0">
         <x:v>154.36</x:v>
@@ -6467,7 +6467,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I149" s="0">
-        <x:v>15</x:v>
+        <x:v>14.51</x:v>
       </x:c>
       <x:c r="J149" s="0">
         <x:v>14.81</x:v>
@@ -6502,7 +6502,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I150" s="0">
-        <x:v>1.24</x:v>
+        <x:v>1.23</x:v>
       </x:c>
       <x:c r="J150" s="0">
         <x:v>13.82</x:v>
@@ -6537,7 +6537,7 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I151" s="0">
-        <x:v>5.77</x:v>
+        <x:v>5.7</x:v>
       </x:c>
       <x:c r="J151" s="0">
         <x:v>7.15</x:v>
@@ -6572,7 +6572,7 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I152" s="0">
-        <x:v>760</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="J152" s="0">
         <x:v>226</x:v>
@@ -6607,7 +6607,7 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I153" s="0">
-        <x:v>545</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="J153" s="0">
         <x:v>242.84</x:v>
@@ -6642,7 +6642,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I154" s="0">
-        <x:v>15</x:v>
+        <x:v>14.51</x:v>
       </x:c>
       <x:c r="J154" s="0">
         <x:v>14.11</x:v>
@@ -6677,7 +6677,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I155" s="0">
-        <x:v>1.24</x:v>
+        <x:v>1.23</x:v>
       </x:c>
       <x:c r="J155" s="0">
         <x:v>14.58</x:v>
@@ -6712,7 +6712,7 @@
         <x:v>1.51</x:v>
       </x:c>
       <x:c r="I156" s="0">
-        <x:v>138.1</x:v>
+        <x:v>143.1</x:v>
       </x:c>
       <x:c r="J156" s="0">
         <x:v>138.67</x:v>
@@ -6747,7 +6747,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I157" s="0">
-        <x:v>288</x:v>
+        <x:v>287.5</x:v>
       </x:c>
       <x:c r="J157" s="0">
         <x:v>0</x:v>
@@ -6779,7 +6779,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I158" s="0">
-        <x:v>3.9</x:v>
+        <x:v>3.89</x:v>
       </x:c>
       <x:c r="J158" s="0">
         <x:v>11.89</x:v>
@@ -6814,7 +6814,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I159" s="0">
-        <x:v>45.92</x:v>
+        <x:v>44.8</x:v>
       </x:c>
       <x:c r="J159" s="0">
         <x:v>94</x:v>
@@ -6849,7 +6849,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I160" s="0">
-        <x:v>7.02</x:v>
+        <x:v>6.99</x:v>
       </x:c>
       <x:c r="J160" s="0">
         <x:v>7.7</x:v>
@@ -6884,7 +6884,7 @@
         <x:v>0.22</x:v>
       </x:c>
       <x:c r="I161" s="0">
-        <x:v>3.21</x:v>
+        <x:v>3.1</x:v>
       </x:c>
       <x:c r="J161" s="0">
         <x:v>1.6</x:v>
@@ -6919,7 +6919,7 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I162" s="0">
-        <x:v>4.14</x:v>
+        <x:v>4.07</x:v>
       </x:c>
       <x:c r="J162" s="0">
         <x:v>19.21</x:v>
@@ -6954,7 +6954,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I163" s="0">
-        <x:v>18.16</x:v>
+        <x:v>17.87</x:v>
       </x:c>
       <x:c r="J163" s="0">
         <x:v>23.4</x:v>
@@ -6989,7 +6989,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="I164" s="0">
-        <x:v>2.56</x:v>
+        <x:v>2.45</x:v>
       </x:c>
       <x:c r="J164" s="0">
         <x:v>7.44</x:v>
@@ -7024,7 +7024,7 @@
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="I165" s="0">
-        <x:v>23.4</x:v>
+        <x:v>23.38</x:v>
       </x:c>
       <x:c r="J165" s="0">
         <x:v>51.7</x:v>
@@ -7059,7 +7059,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I166" s="0">
-        <x:v>2.23</x:v>
+        <x:v>2.24</x:v>
       </x:c>
       <x:c r="J166" s="0">
         <x:v>26.8</x:v>
@@ -7094,7 +7094,7 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="I167" s="0">
-        <x:v>39.94</x:v>
+        <x:v>39.3</x:v>
       </x:c>
       <x:c r="J167" s="0">
         <x:v>66.95</x:v>
@@ -7129,7 +7129,7 @@
         <x:v>0.44</x:v>
       </x:c>
       <x:c r="I168" s="0">
-        <x:v>220.9</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="J168" s="0">
         <x:v>57.32</x:v>
@@ -7164,7 +7164,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I169" s="0">
-        <x:v>2.73</x:v>
+        <x:v>2.77</x:v>
       </x:c>
       <x:c r="J169" s="0">
         <x:v>4.26</x:v>
@@ -7199,7 +7199,7 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I170" s="0">
-        <x:v>8.42</x:v>
+        <x:v>8.46</x:v>
       </x:c>
       <x:c r="J170" s="0">
         <x:v>63.77</x:v>
@@ -7234,7 +7234,7 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I171" s="0">
-        <x:v>10.69</x:v>
+        <x:v>10.6</x:v>
       </x:c>
       <x:c r="J171" s="0">
         <x:v>13.33</x:v>
@@ -7269,7 +7269,7 @@
         <x:v>2.71</x:v>
       </x:c>
       <x:c r="I172" s="0">
-        <x:v>7.24</x:v>
+        <x:v>7.12</x:v>
       </x:c>
       <x:c r="J172" s="0">
         <x:v>5.82</x:v>
@@ -7304,7 +7304,7 @@
         <x:v>0.66</x:v>
       </x:c>
       <x:c r="I173" s="0">
-        <x:v>5.77</x:v>
+        <x:v>5.68</x:v>
       </x:c>
       <x:c r="J173" s="0">
         <x:v>14.27</x:v>

</xml_diff>

<commit_message>
Site guncellemesi - 11.09.2026 18:35
</commit_message>
<xml_diff>
--- a/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
+++ b/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
@@ -82,6 +82,9 @@
     <x:t>01.09.2026</x:t>
   </x:si>
   <x:si>
+    <x:t>10.09.2026</x:t>
+  </x:si>
+  <x:si>
     <x:t>SUWEN</x:t>
   </x:si>
   <x:si>
@@ -130,27 +133,27 @@
     <x:t>04.08.2026</x:t>
   </x:si>
   <x:si>
+    <x:t>OTTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>03.08.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>REEDR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>07.08.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKSGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>31.07.2026</x:t>
+  </x:si>
+  <x:si>
     <x:t>26.08.2026</x:t>
   </x:si>
   <x:si>
-    <x:t>OTTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>03.08.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>REEDR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>07.08.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>31.07.2026</x:t>
-  </x:si>
-  <x:si>
     <x:t>31.08.2026</x:t>
   </x:si>
   <x:si>
@@ -178,286 +181,286 @@
     <x:t>14.07.2026</x:t>
   </x:si>
   <x:si>
+    <x:t>ARSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10.07.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIMAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>03.07.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BALAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEREL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30.06.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRALT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>29.06.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12.08.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAGEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12.06.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11.09.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLSYN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04.05.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11.12.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BOBET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27.04.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14.04.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YYLGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22.04.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>18.08.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALBRK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>METRO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06.04.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>29.07.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARMGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>31.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EFOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>25.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GWIND</x:t>
+  </x:si>
+  <x:si>
+    <x:t>24.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05.05.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KONKA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>03.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HLGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09.02.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEPET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27.01.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>23.01.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19.01.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MIATK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>17.12.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLYPV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09.12.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIGCH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04.12.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BTCIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02.12.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LIDER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27.11.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DAGI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20.11.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GIPTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15.11.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05.12.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOKNR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14.11.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19.11.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06.11.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06.10.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESCAR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>29.09.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13.03.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12.09.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>29.08.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>28.08.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>03.10.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22.08.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06.08.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MERCN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21.08.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22.07.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>31.07.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>08.07.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>24.07.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CWENE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02.07.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BORLS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20.06.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>17.09.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAVI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10.06.2025</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21.05.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORGE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27.05.2025</x:t>
+  </x:si>
+  <x:si>
     <x:t>09.09.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10.07.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>03.07.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BALAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEREL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>30.06.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRALT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>29.06.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12.08.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAGEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12.06.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10.09.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSYN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04.05.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11.12.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BOBET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27.04.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14.04.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YYLGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22.04.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>18.08.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALBRK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>METRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>06.04.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>29.07.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARMGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>31.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EFOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>25.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GWIND</x:t>
-  </x:si>
-  <x:si>
-    <x:t>24.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>05.05.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KONKA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>03.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HLGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>09.02.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEPET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27.01.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>23.01.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>19.01.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MIATK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>17.12.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLYPV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>09.12.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>09.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIGCH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04.12.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>04.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BTCIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02.12.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LIDER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27.11.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DAGI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20.11.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GIPTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>15.11.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>05.12.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOKNR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14.11.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>19.11.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>06.11.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>06.10.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESCAR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>29.09.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>13.03.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12.09.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>29.08.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>28.08.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>03.10.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22.08.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>06.08.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MERCN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21.08.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22.07.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>31.07.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>08.07.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>24.07.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CWENE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02.07.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BORLS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20.06.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>17.09.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAVI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10.06.2025</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21.05.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORGE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27.05.2025</x:t>
   </x:si>
   <x:si>
     <x:t>MOPAS</x:t>
@@ -1421,7 +1424,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>8.68</x:v>
+        <x:v>8.73</x:v>
       </x:c>
       <x:c r="J2" s="0">
         <x:v>0</x:v>
@@ -1453,7 +1456,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>5.15</x:v>
+        <x:v>4.88</x:v>
       </x:c>
       <x:c r="J3" s="0">
         <x:v>0</x:v>
@@ -1485,7 +1488,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>6.66</x:v>
+        <x:v>6.45</x:v>
       </x:c>
       <x:c r="J4" s="0">
         <x:v>0</x:v>
@@ -1517,7 +1520,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>9.2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="J5" s="0">
         <x:v>8.74</x:v>
@@ -1533,8 +1536,8 @@
       <x:c r="B6" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>13</x:v>
+      <x:c r="C6" s="0">
+        <x:v>100000</x:v>
       </x:c>
       <x:c r="D6" s="0">
         <x:v>13500000</x:v>
@@ -1542,25 +1545,28 @@
       <x:c r="E6" s="0">
         <x:v>400000000</x:v>
       </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>13</x:v>
+      <x:c r="F6" s="0">
+        <x:v>2503000</x:v>
       </x:c>
       <x:c r="G6" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>0</x:v>
+        <x:v>0.05</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>26.1</x:v>
+        <x:v>25.36</x:v>
       </x:c>
       <x:c r="J6" s="0">
-        <x:v>0</x:v>
+        <x:v>25.03</x:v>
+      </x:c>
+      <x:c r="K6" s="0" t="s">
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:11">
       <x:c r="A7" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>21</x:v>
@@ -1584,7 +1590,7 @@
         <x:v>3.7</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>6.67</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>6.99</x:v>
@@ -1595,7 +1601,7 @@
     </x:row>
     <x:row r="8" spans="1:11">
       <x:c r="A8" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>21</x:v>
@@ -1619,7 +1625,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>21.22</x:v>
+        <x:v>20.84</x:v>
       </x:c>
       <x:c r="J8" s="0">
         <x:v>23.68</x:v>
@@ -1630,10 +1636,10 @@
     </x:row>
     <x:row r="9" spans="1:11">
       <x:c r="A9" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C9" s="0">
         <x:v>1000000</x:v>
@@ -1654,21 +1660,21 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>7.12</x:v>
+        <x:v>7.06</x:v>
       </x:c>
       <x:c r="J9" s="0">
         <x:v>8.39</x:v>
       </x:c>
       <x:c r="K9" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:11">
       <x:c r="A10" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C10" s="0">
         <x:v>2300000</x:v>
@@ -1689,21 +1695,21 @@
         <x:v>3.83</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>13.75</x:v>
+        <x:v>14.19</x:v>
       </x:c>
       <x:c r="J10" s="0">
         <x:v>0.76</x:v>
       </x:c>
       <x:c r="K10" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:11">
       <x:c r="A11" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C11" s="0">
         <x:v>4790000</x:v>
@@ -1724,21 +1730,21 @@
         <x:v>7.98</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>4.76</x:v>
+        <x:v>4.77</x:v>
       </x:c>
       <x:c r="J11" s="0">
         <x:v>1.47</x:v>
       </x:c>
       <x:c r="K11" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:11">
       <x:c r="A12" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C12" s="0">
         <x:v>4850000</x:v>
@@ -1759,21 +1765,21 @@
         <x:v>8.08</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>14.5</x:v>
+        <x:v>14.4</x:v>
       </x:c>
       <x:c r="J12" s="0">
         <x:v>0.73</x:v>
       </x:c>
       <x:c r="K12" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:11">
       <x:c r="A13" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C13" s="0">
         <x:v>61493</x:v>
@@ -1794,7 +1800,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>66.5</x:v>
+        <x:v>66.1</x:v>
       </x:c>
       <x:c r="J13" s="0">
         <x:v>64.98</x:v>
@@ -1805,13 +1811,13 @@
     </x:row>
     <x:row r="14" spans="1:11">
       <x:c r="A14" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>10000000</x:v>
+        <x:v>20000000</x:v>
       </x:c>
       <x:c r="D14" s="0">
         <x:v>500000000</x:v>
@@ -1820,22 +1826,22 @@
         <x:v>750000000</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>13300000</x:v>
+        <x:v>26500000</x:v>
       </x:c>
       <x:c r="G14" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>0.05</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>1.35</x:v>
+        <x:v>1.34</x:v>
       </x:c>
       <x:c r="J14" s="0">
         <x:v>1.33</x:v>
       </x:c>
       <x:c r="K14" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:11">
@@ -1864,7 +1870,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>136.1</x:v>
+        <x:v>128.7</x:v>
       </x:c>
       <x:c r="J15" s="0">
         <x:v>0</x:v>
@@ -1896,7 +1902,7 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>5.44</x:v>
+        <x:v>5.41</x:v>
       </x:c>
       <x:c r="J16" s="0">
         <x:v>6.13</x:v>
@@ -1931,13 +1937,13 @@
         <x:v>0.43</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>9.93</x:v>
+        <x:v>10.2</x:v>
       </x:c>
       <x:c r="J17" s="0">
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="K17" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:11">
@@ -1966,21 +1972,21 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>9.2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="J18" s="0">
         <x:v>9.69</x:v>
       </x:c>
       <x:c r="K18" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:11">
       <x:c r="A19" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
         <x:v>13</x:v>
@@ -2001,7 +2007,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>18.44</x:v>
+        <x:v>18.29</x:v>
       </x:c>
       <x:c r="J19" s="0">
         <x:v>0</x:v>
@@ -2009,10 +2015,10 @@
     </x:row>
     <x:row r="20" spans="1:11">
       <x:c r="A20" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B20" s="0" t="s">
         <x:v>48</x:v>
-      </x:c>
-      <x:c r="B20" s="0" t="s">
-        <x:v>47</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
         <x:v>13</x:v>
@@ -2041,10 +2047,10 @@
     </x:row>
     <x:row r="21" spans="1:11">
       <x:c r="A21" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C21" s="0">
         <x:v>200000</x:v>
@@ -2065,24 +2071,24 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>16.12</x:v>
+        <x:v>17.13</x:v>
       </x:c>
       <x:c r="J21" s="0">
         <x:v>15.87</x:v>
       </x:c>
       <x:c r="K21" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:11">
       <x:c r="A22" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C22" s="0">
-        <x:v>4540000</x:v>
+        <x:v>5017182</x:v>
       </x:c>
       <x:c r="D22" s="0">
         <x:v>40000000</x:v>
@@ -2091,22 +2097,22 @@
         <x:v>1000000000</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>86614200</x:v>
+        <x:v>95092049</x:v>
       </x:c>
       <x:c r="G22" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>0.55</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>17.85</x:v>
+        <x:v>17.89</x:v>
       </x:c>
       <x:c r="J22" s="0">
-        <x:v>19.08</x:v>
+        <x:v>18.95</x:v>
       </x:c>
       <x:c r="K22" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:11">
@@ -2135,7 +2141,7 @@
         <x:v>0.65</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>4.01</x:v>
+        <x:v>4.08</x:v>
       </x:c>
       <x:c r="J23" s="0">
         <x:v>3.49</x:v>
@@ -2170,13 +2176,13 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>430</x:v>
+        <x:v>434.75</x:v>
       </x:c>
       <x:c r="J24" s="0">
         <x:v>380.17</x:v>
       </x:c>
       <x:c r="K24" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:11">
@@ -2187,7 +2193,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="C25" s="0">
-        <x:v>178529</x:v>
+        <x:v>179529</x:v>
       </x:c>
       <x:c r="D25" s="0">
         <x:v>230000</x:v>
@@ -2196,7 +2202,7 @@
         <x:v>15000000</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>12460563</x:v>
+        <x:v>12528563</x:v>
       </x:c>
       <x:c r="G25" s="0">
         <x:v>1.66</x:v>
@@ -2205,13 +2211,13 @@
         <x:v>1.29</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>70.65</x:v>
+        <x:v>69.25</x:v>
       </x:c>
       <x:c r="J25" s="0">
-        <x:v>69.8</x:v>
+        <x:v>69.79</x:v>
       </x:c>
       <x:c r="K25" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:11">
@@ -2240,13 +2246,13 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>38.62</x:v>
+        <x:v>36.2</x:v>
       </x:c>
       <x:c r="J26" s="0">
         <x:v>38.82</x:v>
       </x:c>
       <x:c r="K26" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:11">
@@ -2275,7 +2281,7 @@
         <x:v>1.8</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>52.45</x:v>
+        <x:v>53.65</x:v>
       </x:c>
       <x:c r="J27" s="0">
         <x:v>48.23</x:v>
@@ -2292,7 +2298,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="C28" s="0">
-        <x:v>48947313</x:v>
+        <x:v>49697313</x:v>
       </x:c>
       <x:c r="D28" s="0">
         <x:v>25000000</x:v>
@@ -2301,19 +2307,19 @@
         <x:v>1000000000</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>1674316254</x:v>
+        <x:v>1701868254</x:v>
       </x:c>
       <x:c r="G28" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.66</x:v>
+        <x:v>1.68</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>37.24</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="J28" s="0">
-        <x:v>34.21</x:v>
+        <x:v>34.24</x:v>
       </x:c>
       <x:c r="K28" s="0" t="s">
         <x:v>67</x:v>
@@ -2345,7 +2351,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>16.32</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="J29" s="0">
         <x:v>5.49</x:v>
@@ -2380,7 +2386,7 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>23.62</x:v>
+        <x:v>24.72</x:v>
       </x:c>
       <x:c r="J30" s="0">
         <x:v>21.09</x:v>
@@ -2415,7 +2421,7 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>10.11</x:v>
+        <x:v>10.1</x:v>
       </x:c>
       <x:c r="J31" s="0">
         <x:v>10.31</x:v>
@@ -2450,7 +2456,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I32" s="0">
-        <x:v>9.21</x:v>
+        <x:v>9.15</x:v>
       </x:c>
       <x:c r="J32" s="0">
         <x:v>0</x:v>
@@ -2482,7 +2488,7 @@
         <x:v>0.35</x:v>
       </x:c>
       <x:c r="I33" s="0">
-        <x:v>8.4</x:v>
+        <x:v>8.67</x:v>
       </x:c>
       <x:c r="J33" s="0">
         <x:v>7.46</x:v>
@@ -2517,7 +2523,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I34" s="0">
-        <x:v>191</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="J34" s="0">
         <x:v>0</x:v>
@@ -2549,7 +2555,7 @@
         <x:v>0.82</x:v>
       </x:c>
       <x:c r="I35" s="0">
-        <x:v>18.8</x:v>
+        <x:v>20.06</x:v>
       </x:c>
       <x:c r="J35" s="0">
         <x:v>7.13</x:v>
@@ -2584,7 +2590,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I36" s="0">
-        <x:v>23.14</x:v>
+        <x:v>22.98</x:v>
       </x:c>
       <x:c r="J36" s="0">
         <x:v>28.89</x:v>
@@ -2619,7 +2625,7 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I37" s="0">
-        <x:v>9.52</x:v>
+        <x:v>9.33</x:v>
       </x:c>
       <x:c r="J37" s="0">
         <x:v>15.08</x:v>
@@ -2654,7 +2660,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I38" s="0">
-        <x:v>4.55</x:v>
+        <x:v>4.48</x:v>
       </x:c>
       <x:c r="J38" s="0">
         <x:v>0</x:v>
@@ -2686,13 +2692,13 @@
         <x:v>2.78</x:v>
       </x:c>
       <x:c r="I39" s="0">
-        <x:v>21.26</x:v>
+        <x:v>20.72</x:v>
       </x:c>
       <x:c r="J39" s="0">
         <x:v>23.25</x:v>
       </x:c>
       <x:c r="K39" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:11">
@@ -2703,7 +2709,7 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="C40" s="0">
-        <x:v>28921768</x:v>
+        <x:v>28952670</x:v>
       </x:c>
       <x:c r="D40" s="0">
         <x:v>80000000</x:v>
@@ -2712,7 +2718,7 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F40" s="0">
-        <x:v>809671512</x:v>
+        <x:v>810882777</x:v>
       </x:c>
       <x:c r="G40" s="0">
         <x:v>0</x:v>
@@ -2721,13 +2727,13 @@
         <x:v>1.11</x:v>
       </x:c>
       <x:c r="I40" s="0">
-        <x:v>39.24</x:v>
+        <x:v>40.54</x:v>
       </x:c>
       <x:c r="J40" s="0">
-        <x:v>28</x:v>
+        <x:v>28.01</x:v>
       </x:c>
       <x:c r="K40" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:11">
@@ -2756,7 +2762,7 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I41" s="0">
-        <x:v>11.27</x:v>
+        <x:v>11.42</x:v>
       </x:c>
       <x:c r="J41" s="0">
         <x:v>13.34</x:v>
@@ -2791,7 +2797,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I42" s="0">
-        <x:v>38.08</x:v>
+        <x:v>37.4</x:v>
       </x:c>
       <x:c r="J42" s="0">
         <x:v>39.18</x:v>
@@ -2826,7 +2832,7 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="I43" s="0">
-        <x:v>63.75</x:v>
+        <x:v>61.7</x:v>
       </x:c>
       <x:c r="J43" s="0">
         <x:v>59.93</x:v>
@@ -2896,7 +2902,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I45" s="0">
-        <x:v>3.92</x:v>
+        <x:v>3.91</x:v>
       </x:c>
       <x:c r="J45" s="0">
         <x:v>0</x:v>
@@ -2928,7 +2934,7 @@
         <x:v>0.43</x:v>
       </x:c>
       <x:c r="I46" s="0">
-        <x:v>22.44</x:v>
+        <x:v>21.58</x:v>
       </x:c>
       <x:c r="J46" s="0">
         <x:v>45.09</x:v>
@@ -2945,7 +2951,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="C47" s="0">
-        <x:v>17473248</x:v>
+        <x:v>17973248</x:v>
       </x:c>
       <x:c r="D47" s="0">
         <x:v>35000000</x:v>
@@ -2954,22 +2960,22 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F47" s="0">
-        <x:v>152638225</x:v>
+        <x:v>157359225</x:v>
       </x:c>
       <x:c r="G47" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H47" s="0">
-        <x:v>4.37</x:v>
+        <x:v>4.49</x:v>
       </x:c>
       <x:c r="I47" s="0">
-        <x:v>9.4</x:v>
+        <x:v>9.16</x:v>
       </x:c>
       <x:c r="J47" s="0">
-        <x:v>8.74</x:v>
+        <x:v>8.76</x:v>
       </x:c>
       <x:c r="K47" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:11">
@@ -2998,7 +3004,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I48" s="0">
-        <x:v>73.5</x:v>
+        <x:v>71.6</x:v>
       </x:c>
       <x:c r="J48" s="0">
         <x:v>61.87</x:v>
@@ -3033,7 +3039,7 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I49" s="0">
-        <x:v>17.87</x:v>
+        <x:v>17.9</x:v>
       </x:c>
       <x:c r="J49" s="0">
         <x:v>21.06</x:v>
@@ -3082,7 +3088,7 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="C51" s="0">
-        <x:v>104378690</x:v>
+        <x:v>104895788</x:v>
       </x:c>
       <x:c r="D51" s="0">
         <x:v>200000000</x:v>
@@ -3091,22 +3097,22 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F51" s="0">
-        <x:v>1020837906</x:v>
+        <x:v>1026744716</x:v>
       </x:c>
       <x:c r="G51" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H51" s="0">
-        <x:v>1.16</x:v>
+        <x:v>1.17</x:v>
       </x:c>
       <x:c r="I51" s="0">
-        <x:v>11.47</x:v>
+        <x:v>12.18</x:v>
       </x:c>
       <x:c r="J51" s="0">
-        <x:v>9.78</x:v>
+        <x:v>9.79</x:v>
       </x:c>
       <x:c r="K51" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:11">
@@ -3135,7 +3141,7 @@
         <x:v>3.29</x:v>
       </x:c>
       <x:c r="I52" s="0">
-        <x:v>43.06</x:v>
+        <x:v>43.54</x:v>
       </x:c>
       <x:c r="J52" s="0">
         <x:v>23.95</x:v>
@@ -3170,7 +3176,7 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I53" s="0">
-        <x:v>430</x:v>
+        <x:v>434.75</x:v>
       </x:c>
       <x:c r="J53" s="0">
         <x:v>528.86</x:v>
@@ -3205,7 +3211,7 @@
         <x:v>0.94</x:v>
       </x:c>
       <x:c r="I54" s="0">
-        <x:v>39.24</x:v>
+        <x:v>40.54</x:v>
       </x:c>
       <x:c r="J54" s="0">
         <x:v>24.19</x:v>
@@ -3240,7 +3246,7 @@
         <x:v>0.52</x:v>
       </x:c>
       <x:c r="I55" s="0">
-        <x:v>11.47</x:v>
+        <x:v>12.18</x:v>
       </x:c>
       <x:c r="J55" s="0">
         <x:v>10.74</x:v>
@@ -3275,7 +3281,7 @@
         <x:v>0.69</x:v>
       </x:c>
       <x:c r="I56" s="0">
-        <x:v>6.66</x:v>
+        <x:v>6.45</x:v>
       </x:c>
       <x:c r="J56" s="0">
         <x:v>6.01</x:v>
@@ -3310,13 +3316,13 @@
         <x:v>1.36</x:v>
       </x:c>
       <x:c r="I57" s="0">
-        <x:v>18.6</x:v>
+        <x:v>18.96</x:v>
       </x:c>
       <x:c r="J57" s="0">
         <x:v>25.45</x:v>
       </x:c>
       <x:c r="K57" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:11">
@@ -3345,7 +3351,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I58" s="0">
-        <x:v>4.06</x:v>
+        <x:v>3.99</x:v>
       </x:c>
       <x:c r="J58" s="0">
         <x:v>4.46</x:v>
@@ -3356,7 +3362,7 @@
     </x:row>
     <x:row r="59" spans="1:11">
       <x:c r="A59" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
         <x:v>136</x:v>
@@ -3380,7 +3386,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I59" s="0">
-        <x:v>6.67</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="J59" s="0">
         <x:v>12.82</x:v>
@@ -3415,7 +3421,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I60" s="0">
-        <x:v>31.02</x:v>
+        <x:v>30.22</x:v>
       </x:c>
       <x:c r="J60" s="0">
         <x:v>0</x:v>
@@ -3482,7 +3488,7 @@
         <x:v>1.83</x:v>
       </x:c>
       <x:c r="I62" s="0">
-        <x:v>36.8</x:v>
+        <x:v>37.5</x:v>
       </x:c>
       <x:c r="J62" s="0">
         <x:v>39.62</x:v>
@@ -3517,21 +3523,21 @@
         <x:v>0.95</x:v>
       </x:c>
       <x:c r="I63" s="0">
-        <x:v>23.38</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J63" s="0">
         <x:v>46.8</x:v>
       </x:c>
       <x:c r="K63" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>148</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:11">
       <x:c r="A64" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B64" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C64" s="0" t="s">
         <x:v>13</x:v>
@@ -3552,7 +3558,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I64" s="0">
-        <x:v>25.84</x:v>
+        <x:v>25.36</x:v>
       </x:c>
       <x:c r="J64" s="0">
         <x:v>0</x:v>
@@ -3560,10 +3566,10 @@
     </x:row>
     <x:row r="65" spans="1:11">
       <x:c r="A65" s="0" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="B65" s="0" t="s">
         <x:v>150</x:v>
-      </x:c>
-      <x:c r="B65" s="0" t="s">
-        <x:v>149</x:v>
       </x:c>
       <x:c r="C65" s="0">
         <x:v>8337681</x:v>
@@ -3584,7 +3590,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I65" s="0">
-        <x:v>3.89</x:v>
+        <x:v>3.78</x:v>
       </x:c>
       <x:c r="J65" s="0">
         <x:v>4.47</x:v>
@@ -3595,10 +3601,10 @@
     </x:row>
     <x:row r="66" spans="1:11">
       <x:c r="A66" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B66" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C66" s="0" t="s">
         <x:v>13</x:v>
@@ -3619,7 +3625,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I66" s="0">
-        <x:v>39.3</x:v>
+        <x:v>38.94</x:v>
       </x:c>
       <x:c r="J66" s="0">
         <x:v>0</x:v>
@@ -3627,10 +3633,10 @@
     </x:row>
     <x:row r="67" spans="1:11">
       <x:c r="A67" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B67" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C67" s="0">
         <x:v>1364000</x:v>
@@ -3651,21 +3657,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I67" s="0">
-        <x:v>299.25</x:v>
+        <x:v>300.25</x:v>
       </x:c>
       <x:c r="J67" s="0">
         <x:v>299.91</x:v>
       </x:c>
       <x:c r="K67" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>155</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:11">
       <x:c r="A68" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B68" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="C68" s="0" t="s">
         <x:v>13</x:v>
@@ -3686,7 +3692,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I68" s="0">
-        <x:v>20.8</x:v>
+        <x:v>20.92</x:v>
       </x:c>
       <x:c r="J68" s="0">
         <x:v>0</x:v>
@@ -3694,10 +3700,10 @@
     </x:row>
     <x:row r="69" spans="1:11">
       <x:c r="A69" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B69" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="C69" s="0">
         <x:v>507440</x:v>
@@ -3718,7 +3724,7 @@
         <x:v>0.54</x:v>
       </x:c>
       <x:c r="I69" s="0">
-        <x:v>287.5</x:v>
+        <x:v>277.75</x:v>
       </x:c>
       <x:c r="J69" s="0">
         <x:v>83</x:v>
@@ -3729,10 +3735,10 @@
     </x:row>
     <x:row r="70" spans="1:11">
       <x:c r="A70" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B70" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="C70" s="0">
         <x:v>2000000</x:v>
@@ -3753,21 +3759,21 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I70" s="0">
-        <x:v>34.58</x:v>
+        <x:v>34.38</x:v>
       </x:c>
       <x:c r="J70" s="0">
         <x:v>40.97</x:v>
       </x:c>
       <x:c r="K70" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="71" spans="1:11">
       <x:c r="A71" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B71" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="C71" s="0">
         <x:v>9854768</x:v>
@@ -3788,7 +3794,7 @@
         <x:v>0.62</x:v>
       </x:c>
       <x:c r="I71" s="0">
-        <x:v>21.22</x:v>
+        <x:v>20.84</x:v>
       </x:c>
       <x:c r="J71" s="0">
         <x:v>23.68</x:v>
@@ -3802,7 +3808,7 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B72" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C72" s="0">
         <x:v>324474</x:v>
@@ -3823,7 +3829,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I72" s="0">
-        <x:v>16.32</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="J72" s="0">
         <x:v>5.49</x:v>
@@ -3834,10 +3840,10 @@
     </x:row>
     <x:row r="73" spans="1:11">
       <x:c r="A73" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B73" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="C73" s="0" t="s">
         <x:v>13</x:v>
@@ -3858,7 +3864,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I73" s="0">
-        <x:v>16.12</x:v>
+        <x:v>17.13</x:v>
       </x:c>
       <x:c r="J73" s="0">
         <x:v>0</x:v>
@@ -3866,10 +3872,10 @@
     </x:row>
     <x:row r="74" spans="1:11">
       <x:c r="A74" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B74" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="C74" s="0" t="s">
         <x:v>13</x:v>
@@ -3890,7 +3896,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I74" s="0">
-        <x:v>5.42</x:v>
+        <x:v>5.46</x:v>
       </x:c>
       <x:c r="J74" s="0">
         <x:v>0</x:v>
@@ -3898,10 +3904,10 @@
     </x:row>
     <x:row r="75" spans="1:11">
       <x:c r="A75" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B75" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C75" s="0">
         <x:v>13000000</x:v>
@@ -3922,21 +3928,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I75" s="0">
-        <x:v>6.6</x:v>
+        <x:v>6.54</x:v>
       </x:c>
       <x:c r="J75" s="0">
         <x:v>6.6</x:v>
       </x:c>
       <x:c r="K75" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
     </x:row>
     <x:row r="76" spans="1:11">
       <x:c r="A76" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B76" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C76" s="0">
         <x:v>174500000</x:v>
@@ -3957,13 +3963,13 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I76" s="0">
-        <x:v>2.77</x:v>
+        <x:v>2.82</x:v>
       </x:c>
       <x:c r="J76" s="0">
         <x:v>3.98</x:v>
       </x:c>
       <x:c r="K76" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="77" spans="1:11">
@@ -3971,7 +3977,7 @@
         <x:v>131</x:v>
       </x:c>
       <x:c r="B77" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="C77" s="0">
         <x:v>635229</x:v>
@@ -3992,21 +3998,21 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I77" s="0">
-        <x:v>18.6</x:v>
+        <x:v>18.96</x:v>
       </x:c>
       <x:c r="J77" s="0">
         <x:v>17.83</x:v>
       </x:c>
       <x:c r="K77" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="78" spans="1:11">
       <x:c r="A78" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B78" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C78" s="0">
         <x:v>130000</x:v>
@@ -4027,21 +4033,21 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I78" s="0">
-        <x:v>29.74</x:v>
+        <x:v>31.38</x:v>
       </x:c>
       <x:c r="J78" s="0">
         <x:v>38.06</x:v>
       </x:c>
       <x:c r="K78" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="79" spans="1:11">
       <x:c r="A79" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="B79" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="C79" s="0" t="s">
         <x:v>13</x:v>
@@ -4062,7 +4068,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I79" s="0">
-        <x:v>225</x:v>
+        <x:v>223.8</x:v>
       </x:c>
       <x:c r="J79" s="0">
         <x:v>0</x:v>
@@ -4070,10 +4076,10 @@
     </x:row>
     <x:row r="80" spans="1:11">
       <x:c r="A80" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B80" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="C80" s="0">
         <x:v>447761</x:v>
@@ -4094,21 +4100,21 @@
         <x:v>0.86</x:v>
       </x:c>
       <x:c r="I80" s="0">
-        <x:v>33.84</x:v>
+        <x:v>33.74</x:v>
       </x:c>
       <x:c r="J80" s="0">
         <x:v>41.13</x:v>
       </x:c>
       <x:c r="K80" s="0" t="s">
-        <x:v>179</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="81" spans="1:11">
       <x:c r="A81" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B81" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C81" s="0">
         <x:v>200000</x:v>
@@ -4129,21 +4135,21 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I81" s="0">
-        <x:v>4.58</x:v>
+        <x:v>4.41</x:v>
       </x:c>
       <x:c r="J81" s="0">
         <x:v>20.11</x:v>
       </x:c>
       <x:c r="K81" s="0" t="s">
-        <x:v>182</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="82" spans="1:11">
       <x:c r="A82" s="0" t="s">
-        <x:v>183</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B82" s="0" t="s">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C82" s="0">
         <x:v>946718</x:v>
@@ -4164,21 +4170,21 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I82" s="0">
-        <x:v>46.9</x:v>
+        <x:v>46.88</x:v>
       </x:c>
       <x:c r="J82" s="0">
         <x:v>39.43</x:v>
       </x:c>
       <x:c r="K82" s="0" t="s">
-        <x:v>185</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="83" spans="1:11">
       <x:c r="A83" s="0" t="s">
-        <x:v>186</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B83" s="0" t="s">
-        <x:v>187</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="C83" s="0" t="s">
         <x:v>13</x:v>
@@ -4199,7 +4205,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I83" s="0">
-        <x:v>19.06</x:v>
+        <x:v>19.32</x:v>
       </x:c>
       <x:c r="J83" s="0">
         <x:v>0</x:v>
@@ -4207,10 +4213,10 @@
     </x:row>
     <x:row r="84" spans="1:11">
       <x:c r="A84" s="0" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B84" s="0" t="s">
         <x:v>188</x:v>
-      </x:c>
-      <x:c r="B84" s="0" t="s">
-        <x:v>187</x:v>
       </x:c>
       <x:c r="C84" s="0">
         <x:v>3043115</x:v>
@@ -4231,21 +4237,21 @@
         <x:v>0.12</x:v>
       </x:c>
       <x:c r="I84" s="0">
-        <x:v>21.64</x:v>
+        <x:v>21.88</x:v>
       </x:c>
       <x:c r="J84" s="0">
         <x:v>16.34</x:v>
       </x:c>
       <x:c r="K84" s="0" t="s">
-        <x:v>189</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="85" spans="1:11">
       <x:c r="A85" s="0" t="s">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B85" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C85" s="0">
         <x:v>2382736</x:v>
@@ -4266,21 +4272,21 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="I85" s="0">
-        <x:v>72.3</x:v>
+        <x:v>72.65</x:v>
       </x:c>
       <x:c r="J85" s="0">
         <x:v>38.88</x:v>
       </x:c>
       <x:c r="K85" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="86" spans="1:11">
       <x:c r="A86" s="0" t="s">
-        <x:v>193</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B86" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C86" s="0" t="s">
         <x:v>13</x:v>
@@ -4301,7 +4307,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I86" s="0">
-        <x:v>54.1</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="J86" s="0">
         <x:v>0</x:v>
@@ -4309,10 +4315,10 @@
     </x:row>
     <x:row r="87" spans="1:11">
       <x:c r="A87" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B87" s="0" t="s">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="C87" s="0">
         <x:v>4650000</x:v>
@@ -4333,21 +4339,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I87" s="0">
-        <x:v>11.94</x:v>
+        <x:v>12.05</x:v>
       </x:c>
       <x:c r="J87" s="0">
         <x:v>10.75</x:v>
       </x:c>
       <x:c r="K87" s="0" t="s">
-        <x:v>196</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="88" spans="1:11">
       <x:c r="A88" s="0" t="s">
-        <x:v>197</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="B88" s="0" t="s">
-        <x:v>198</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C88" s="0">
         <x:v>806343</x:v>
@@ -4368,21 +4374,21 @@
         <x:v>2.16</x:v>
       </x:c>
       <x:c r="I88" s="0">
-        <x:v>34.26</x:v>
+        <x:v>34.68</x:v>
       </x:c>
       <x:c r="J88" s="0">
         <x:v>37.66</x:v>
       </x:c>
       <x:c r="K88" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="89" spans="1:11">
       <x:c r="A89" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B89" s="0" t="s">
-        <x:v>198</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C89" s="0">
         <x:v>310000</x:v>
@@ -4403,13 +4409,13 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I89" s="0">
-        <x:v>11.94</x:v>
+        <x:v>12.05</x:v>
       </x:c>
       <x:c r="J89" s="0">
         <x:v>161.23</x:v>
       </x:c>
       <x:c r="K89" s="0" t="s">
-        <x:v>196</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="90" spans="1:11">
@@ -4417,7 +4423,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B90" s="0" t="s">
-        <x:v>198</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C90" s="0">
         <x:v>2000000</x:v>
@@ -4438,7 +4444,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="I90" s="0">
-        <x:v>9.2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="J90" s="0">
         <x:v>15.68</x:v>
@@ -4449,10 +4455,10 @@
     </x:row>
     <x:row r="91" spans="1:11">
       <x:c r="A91" s="0" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="B91" s="0" t="s">
         <x:v>199</x:v>
-      </x:c>
-      <x:c r="B91" s="0" t="s">
-        <x:v>198</x:v>
       </x:c>
       <x:c r="C91" s="0">
         <x:v>1250000</x:v>
@@ -4473,21 +4479,21 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I91" s="0">
-        <x:v>1.95</x:v>
+        <x:v>1.94</x:v>
       </x:c>
       <x:c r="J91" s="0">
         <x:v>8.95</x:v>
       </x:c>
       <x:c r="K91" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="92" spans="1:11">
       <x:c r="A92" s="0" t="s">
-        <x:v>200</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B92" s="0" t="s">
-        <x:v>198</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C92" s="0" t="s">
         <x:v>13</x:v>
@@ -4508,7 +4514,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I92" s="0">
-        <x:v>3.94</x:v>
+        <x:v>3.89</x:v>
       </x:c>
       <x:c r="J92" s="0">
         <x:v>0</x:v>
@@ -4516,10 +4522,10 @@
     </x:row>
     <x:row r="93" spans="1:11">
       <x:c r="A93" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="B93" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C93" s="0">
         <x:v>12500000</x:v>
@@ -4540,21 +4546,21 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="I93" s="0">
-        <x:v>2.05</x:v>
+        <x:v>2.07</x:v>
       </x:c>
       <x:c r="J93" s="0">
         <x:v>4.93</x:v>
       </x:c>
       <x:c r="K93" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="94" spans="1:11">
       <x:c r="A94" s="0" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="B94" s="0" t="s">
         <x:v>203</x:v>
-      </x:c>
-      <x:c r="B94" s="0" t="s">
-        <x:v>202</x:v>
       </x:c>
       <x:c r="C94" s="0">
         <x:v>2093944</x:v>
@@ -4575,21 +4581,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I94" s="0">
-        <x:v>101.6</x:v>
+        <x:v>103.7</x:v>
       </x:c>
       <x:c r="J94" s="0">
         <x:v>95.58</x:v>
       </x:c>
       <x:c r="K94" s="0" t="s">
-        <x:v>204</x:v>
+        <x:v>205</x:v>
       </x:c>
     </x:row>
     <x:row r="95" spans="1:11">
       <x:c r="A95" s="0" t="s">
-        <x:v>205</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="B95" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C95" s="0" t="s">
         <x:v>13</x:v>
@@ -4610,7 +4616,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I95" s="0">
-        <x:v>50.05</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="J95" s="0">
         <x:v>0</x:v>
@@ -4618,10 +4624,10 @@
     </x:row>
     <x:row r="96" spans="1:11">
       <x:c r="A96" s="0" t="s">
-        <x:v>206</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="B96" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C96" s="0">
         <x:v>51245979</x:v>
@@ -4653,10 +4659,10 @@
     </x:row>
     <x:row r="97" spans="1:11">
       <x:c r="A97" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B97" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C97" s="0">
         <x:v>1584837</x:v>
@@ -4677,13 +4683,13 @@
         <x:v>1.08</x:v>
       </x:c>
       <x:c r="I97" s="0">
-        <x:v>66.5</x:v>
+        <x:v>66.1</x:v>
       </x:c>
       <x:c r="J97" s="0">
         <x:v>58.33</x:v>
       </x:c>
       <x:c r="K97" s="0" t="s">
-        <x:v>207</x:v>
+        <x:v>208</x:v>
       </x:c>
     </x:row>
     <x:row r="98" spans="1:11">
@@ -4691,7 +4697,7 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B98" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C98" s="0">
         <x:v>7999148</x:v>
@@ -4712,7 +4718,7 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I98" s="0">
-        <x:v>23.62</x:v>
+        <x:v>24.72</x:v>
       </x:c>
       <x:c r="J98" s="0">
         <x:v>21.09</x:v>
@@ -4723,10 +4729,10 @@
     </x:row>
     <x:row r="99" spans="1:11">
       <x:c r="A99" s="0" t="s">
-        <x:v>208</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B99" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C99" s="0">
         <x:v>14000000</x:v>
@@ -4747,7 +4753,7 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I99" s="0">
-        <x:v>27.88</x:v>
+        <x:v>25.42</x:v>
       </x:c>
       <x:c r="J99" s="0">
         <x:v>16.87</x:v>
@@ -4761,7 +4767,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B100" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C100" s="0">
         <x:v>1700005</x:v>
@@ -4782,21 +4788,21 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I100" s="0">
-        <x:v>5.44</x:v>
+        <x:v>5.41</x:v>
       </x:c>
       <x:c r="J100" s="0">
         <x:v>11.99</x:v>
       </x:c>
       <x:c r="K100" s="0" t="s">
-        <x:v>209</x:v>
+        <x:v>210</x:v>
       </x:c>
     </x:row>
     <x:row r="101" spans="1:11">
       <x:c r="A101" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="B101" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C101" s="0">
         <x:v>6000000</x:v>
@@ -4817,21 +4823,21 @@
         <x:v>0.16</x:v>
       </x:c>
       <x:c r="I101" s="0">
-        <x:v>17.53</x:v>
+        <x:v>16.48</x:v>
       </x:c>
       <x:c r="J101" s="0">
         <x:v>22.05</x:v>
       </x:c>
       <x:c r="K101" s="0" t="s">
-        <x:v>212</x:v>
+        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="102" spans="1:11">
       <x:c r="A102" s="0" t="s">
-        <x:v>213</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B102" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C102" s="0">
         <x:v>1675000</x:v>
@@ -4852,21 +4858,21 @@
         <x:v>1.45</x:v>
       </x:c>
       <x:c r="I102" s="0">
-        <x:v>82</x:v>
+        <x:v>80.6</x:v>
       </x:c>
       <x:c r="J102" s="0">
         <x:v>68.15</x:v>
       </x:c>
       <x:c r="K102" s="0" t="s">
-        <x:v>214</x:v>
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="103" spans="1:11">
       <x:c r="A103" s="0" t="s">
-        <x:v>215</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B103" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C103" s="0">
         <x:v>1824868</x:v>
@@ -4887,7 +4893,7 @@
         <x:v>0.68</x:v>
       </x:c>
       <x:c r="I103" s="0">
-        <x:v>30.5</x:v>
+        <x:v>31.82</x:v>
       </x:c>
       <x:c r="J103" s="0">
         <x:v>35.38</x:v>
@@ -4898,10 +4904,10 @@
     </x:row>
     <x:row r="104" spans="1:11">
       <x:c r="A104" s="0" t="s">
-        <x:v>216</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B104" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C104" s="0" t="s">
         <x:v>13</x:v>
@@ -4922,7 +4928,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I104" s="0">
-        <x:v>6.83</x:v>
+        <x:v>6.77</x:v>
       </x:c>
       <x:c r="J104" s="0">
         <x:v>0</x:v>
@@ -4930,10 +4936,10 @@
     </x:row>
     <x:row r="105" spans="1:11">
       <x:c r="A105" s="0" t="s">
-        <x:v>217</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="B105" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C105" s="0">
         <x:v>1000000</x:v>
@@ -4954,21 +4960,21 @@
         <x:v>0.27</x:v>
       </x:c>
       <x:c r="I105" s="0">
-        <x:v>8.94</x:v>
+        <x:v>9.08</x:v>
       </x:c>
       <x:c r="J105" s="0">
         <x:v>19.79</x:v>
       </x:c>
       <x:c r="K105" s="0" t="s">
-        <x:v>218</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="106" spans="1:11">
       <x:c r="A106" s="0" t="s">
-        <x:v>219</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B106" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C106" s="0">
         <x:v>98551</x:v>
@@ -4989,21 +4995,21 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I106" s="0">
-        <x:v>10.79</x:v>
+        <x:v>10.62</x:v>
       </x:c>
       <x:c r="J106" s="0">
         <x:v>13.15</x:v>
       </x:c>
       <x:c r="K106" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="107" spans="1:11">
       <x:c r="A107" s="0" t="s">
-        <x:v>220</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B107" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C107" s="0">
         <x:v>6049315</x:v>
@@ -5024,21 +5030,21 @@
         <x:v>0.92</x:v>
       </x:c>
       <x:c r="I107" s="0">
-        <x:v>11.29</x:v>
+        <x:v>11.26</x:v>
       </x:c>
       <x:c r="J107" s="0">
         <x:v>10.98</x:v>
       </x:c>
       <x:c r="K107" s="0" t="s">
-        <x:v>221</x:v>
+        <x:v>222</x:v>
       </x:c>
     </x:row>
     <x:row r="108" spans="1:11">
       <x:c r="A108" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B108" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C108" s="0">
         <x:v>37225000</x:v>
@@ -5065,15 +5071,15 @@
         <x:v>4.03</x:v>
       </x:c>
       <x:c r="K108" s="0" t="s">
-        <x:v>196</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="109" spans="1:11">
       <x:c r="A109" s="0" t="s">
-        <x:v>222</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B109" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C109" s="0">
         <x:v>1000000</x:v>
@@ -5094,21 +5100,21 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="I109" s="0">
-        <x:v>219.4</x:v>
+        <x:v>228.8</x:v>
       </x:c>
       <x:c r="J109" s="0">
         <x:v>284.58</x:v>
       </x:c>
       <x:c r="K109" s="0" t="s">
-        <x:v>223</x:v>
+        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="110" spans="1:11">
       <x:c r="A110" s="0" t="s">
-        <x:v>224</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B110" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C110" s="0">
         <x:v>600000</x:v>
@@ -5129,21 +5135,21 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="I110" s="0">
-        <x:v>6.46</x:v>
+        <x:v>5.83</x:v>
       </x:c>
       <x:c r="J110" s="0">
         <x:v>38.02</x:v>
       </x:c>
       <x:c r="K110" s="0" t="s">
-        <x:v>225</x:v>
+        <x:v>226</x:v>
       </x:c>
     </x:row>
     <x:row r="111" spans="1:11">
       <x:c r="A111" s="0" t="s">
-        <x:v>226</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="B111" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C111" s="0">
         <x:v>11703083</x:v>
@@ -5164,21 +5170,21 @@
         <x:v>1.67</x:v>
       </x:c>
       <x:c r="I111" s="0">
-        <x:v>195.8</x:v>
+        <x:v>205.6</x:v>
       </x:c>
       <x:c r="J111" s="0">
         <x:v>83.62</x:v>
       </x:c>
       <x:c r="K111" s="0" t="s">
-        <x:v>227</x:v>
+        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="112" spans="1:11">
       <x:c r="A112" s="0" t="s">
-        <x:v>228</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="B112" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="C112" s="0">
         <x:v>5100000</x:v>
@@ -5199,13 +5205,13 @@
         <x:v>4.31</x:v>
       </x:c>
       <x:c r="I112" s="0">
-        <x:v>30.62</x:v>
+        <x:v>31.4</x:v>
       </x:c>
       <x:c r="J112" s="0">
         <x:v>17.65</x:v>
       </x:c>
       <x:c r="K112" s="0" t="s">
-        <x:v>229</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="113" spans="1:11">
@@ -5213,7 +5219,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B113" s="0" t="s">
-        <x:v>230</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C113" s="0">
         <x:v>3228679</x:v>
@@ -5234,7 +5240,7 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I113" s="0">
-        <x:v>8.68</x:v>
+        <x:v>8.73</x:v>
       </x:c>
       <x:c r="J113" s="0">
         <x:v>15.92</x:v>
@@ -5245,10 +5251,10 @@
     </x:row>
     <x:row r="114" spans="1:11">
       <x:c r="A114" s="0" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="B114" s="0" t="s">
         <x:v>231</x:v>
-      </x:c>
-      <x:c r="B114" s="0" t="s">
-        <x:v>230</x:v>
       </x:c>
       <x:c r="C114" s="0">
         <x:v>150000</x:v>
@@ -5269,21 +5275,21 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I114" s="0">
-        <x:v>5.38</x:v>
+        <x:v>5.39</x:v>
       </x:c>
       <x:c r="J114" s="0">
         <x:v>40.97</x:v>
       </x:c>
       <x:c r="K114" s="0" t="s">
-        <x:v>232</x:v>
+        <x:v>233</x:v>
       </x:c>
     </x:row>
     <x:row r="115" spans="1:11">
       <x:c r="A115" s="0" t="s">
-        <x:v>233</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="B115" s="0" t="s">
-        <x:v>230</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C115" s="0" t="s">
         <x:v>13</x:v>
@@ -5304,7 +5310,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I115" s="0">
-        <x:v>11.18</x:v>
+        <x:v>11.6</x:v>
       </x:c>
       <x:c r="J115" s="0">
         <x:v>0</x:v>
@@ -5312,10 +5318,10 @@
     </x:row>
     <x:row r="116" spans="1:11">
       <x:c r="A116" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="B116" s="0" t="s">
-        <x:v>230</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C116" s="0">
         <x:v>366107</x:v>
@@ -5336,13 +5342,13 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I116" s="0">
-        <x:v>14.64</x:v>
+        <x:v>14.62</x:v>
       </x:c>
       <x:c r="J116" s="0">
         <x:v>16.42</x:v>
       </x:c>
       <x:c r="K116" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="117" spans="1:11">
@@ -5350,7 +5356,7 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="B117" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C117" s="0">
         <x:v>120000</x:v>
@@ -5371,21 +5377,21 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I117" s="0">
-        <x:v>191</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="J117" s="0">
         <x:v>31.92</x:v>
       </x:c>
       <x:c r="K117" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="118" spans="1:11">
       <x:c r="A118" s="0" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="B118" s="0" t="s">
         <x:v>236</x:v>
-      </x:c>
-      <x:c r="B118" s="0" t="s">
-        <x:v>235</x:v>
       </x:c>
       <x:c r="C118" s="0">
         <x:v>13050000</x:v>
@@ -5406,21 +5412,21 @@
         <x:v>3.13</x:v>
       </x:c>
       <x:c r="I118" s="0">
-        <x:v>116.6</x:v>
+        <x:v>117.4</x:v>
       </x:c>
       <x:c r="J118" s="0">
         <x:v>94.36</x:v>
       </x:c>
       <x:c r="K118" s="0" t="s">
-        <x:v>237</x:v>
+        <x:v>238</x:v>
       </x:c>
     </x:row>
     <x:row r="119" spans="1:11">
       <x:c r="A119" s="0" t="s">
-        <x:v>238</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="B119" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C119" s="0">
         <x:v>36605658</x:v>
@@ -5441,13 +5447,13 @@
         <x:v>3.66</x:v>
       </x:c>
       <x:c r="I119" s="0">
-        <x:v>4.68</x:v>
+        <x:v>4.65</x:v>
       </x:c>
       <x:c r="J119" s="0">
         <x:v>4.76</x:v>
       </x:c>
       <x:c r="K119" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="120" spans="1:11">
@@ -5455,7 +5461,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B120" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C120" s="0">
         <x:v>1000000</x:v>
@@ -5476,21 +5482,21 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I120" s="0">
-        <x:v>430</x:v>
+        <x:v>434.75</x:v>
       </x:c>
       <x:c r="J120" s="0">
         <x:v>429.82</x:v>
       </x:c>
       <x:c r="K120" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>203</x:v>
       </x:c>
     </x:row>
     <x:row r="121" spans="1:11">
       <x:c r="A121" s="0" t="s">
-        <x:v>239</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="B121" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C121" s="0">
         <x:v>300000</x:v>
@@ -5511,21 +5517,21 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I121" s="0">
-        <x:v>3.05</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J121" s="0">
         <x:v>2.64</x:v>
       </x:c>
       <x:c r="K121" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="122" spans="1:11">
       <x:c r="A122" s="0" t="s">
-        <x:v>240</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="B122" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C122" s="0">
         <x:v>2175097</x:v>
@@ -5546,21 +5552,21 @@
         <x:v>1.45</x:v>
       </x:c>
       <x:c r="I122" s="0">
-        <x:v>13.16</x:v>
+        <x:v>13.69</x:v>
       </x:c>
       <x:c r="J122" s="0">
         <x:v>8.23</x:v>
       </x:c>
       <x:c r="K122" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="123" spans="1:11">
       <x:c r="A123" s="0" t="s">
-        <x:v>241</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="B123" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C123" s="0" t="s">
         <x:v>13</x:v>
@@ -5581,7 +5587,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I123" s="0">
-        <x:v>2.81</x:v>
+        <x:v>2.76</x:v>
       </x:c>
       <x:c r="J123" s="0">
         <x:v>0</x:v>
@@ -5589,10 +5595,10 @@
     </x:row>
     <x:row r="124" spans="1:11">
       <x:c r="A124" s="0" t="s">
-        <x:v>242</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="B124" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C124" s="0">
         <x:v>43000</x:v>
@@ -5613,21 +5619,21 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I124" s="0">
-        <x:v>27.36</x:v>
+        <x:v>27.46</x:v>
       </x:c>
       <x:c r="J124" s="0">
         <x:v>23.83</x:v>
       </x:c>
       <x:c r="K124" s="0" t="s">
-        <x:v>243</x:v>
+        <x:v>244</x:v>
       </x:c>
     </x:row>
     <x:row r="125" spans="1:11">
       <x:c r="A125" s="0" t="s">
-        <x:v>244</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="B125" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C125" s="0">
         <x:v>9937037</x:v>
@@ -5648,21 +5654,21 @@
         <x:v>0.53</x:v>
       </x:c>
       <x:c r="I125" s="0">
-        <x:v>2.25</x:v>
+        <x:v>2.31</x:v>
       </x:c>
       <x:c r="J125" s="0">
         <x:v>5.03</x:v>
       </x:c>
       <x:c r="K125" s="0" t="s">
-        <x:v>245</x:v>
+        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="126" spans="1:11">
       <x:c r="A126" s="0" t="s">
-        <x:v>246</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="B126" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C126" s="0" t="s">
         <x:v>13</x:v>
@@ -5683,7 +5689,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I126" s="0">
-        <x:v>2.71</x:v>
+        <x:v>2.65</x:v>
       </x:c>
       <x:c r="J126" s="0">
         <x:v>0</x:v>
@@ -5694,7 +5700,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="B127" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C127" s="0">
         <x:v>13064888</x:v>
@@ -5715,13 +5721,13 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I127" s="0">
-        <x:v>39.24</x:v>
+        <x:v>40.54</x:v>
       </x:c>
       <x:c r="J127" s="0">
         <x:v>20.53</x:v>
       </x:c>
       <x:c r="K127" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="128" spans="1:11">
@@ -5729,7 +5735,7 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="B128" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C128" s="0">
         <x:v>111673026</x:v>
@@ -5750,21 +5756,21 @@
         <x:v>1.24</x:v>
       </x:c>
       <x:c r="I128" s="0">
-        <x:v>11.47</x:v>
+        <x:v>12.18</x:v>
       </x:c>
       <x:c r="J128" s="0">
         <x:v>4.48</x:v>
       </x:c>
       <x:c r="K128" s="0" t="s">
-        <x:v>248</x:v>
+        <x:v>249</x:v>
       </x:c>
     </x:row>
     <x:row r="129" spans="1:11">
       <x:c r="A129" s="0" t="s">
-        <x:v>249</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="B129" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C129" s="0" t="s">
         <x:v>13</x:v>
@@ -5785,7 +5791,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I129" s="0">
-        <x:v>3.7</x:v>
+        <x:v>3.65</x:v>
       </x:c>
       <x:c r="J129" s="0">
         <x:v>0</x:v>
@@ -5793,10 +5799,10 @@
     </x:row>
     <x:row r="130" spans="1:11">
       <x:c r="A130" s="0" t="s">
-        <x:v>250</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="B130" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C130" s="0" t="s">
         <x:v>13</x:v>
@@ -5817,7 +5823,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I130" s="0">
-        <x:v>7.08</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="J130" s="0">
         <x:v>0</x:v>
@@ -5825,10 +5831,10 @@
     </x:row>
     <x:row r="131" spans="1:11">
       <x:c r="A131" s="0" t="s">
-        <x:v>251</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="B131" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C131" s="0">
         <x:v>1100000</x:v>
@@ -5849,21 +5855,21 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I131" s="0">
-        <x:v>167</x:v>
+        <x:v>183.7</x:v>
       </x:c>
       <x:c r="J131" s="0">
         <x:v>50.97</x:v>
       </x:c>
       <x:c r="K131" s="0" t="s">
-        <x:v>248</x:v>
+        <x:v>249</x:v>
       </x:c>
     </x:row>
     <x:row r="132" spans="1:11">
       <x:c r="A132" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B132" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C132" s="0">
         <x:v>6598092</x:v>
@@ -5884,21 +5890,21 @@
         <x:v>5.91</x:v>
       </x:c>
       <x:c r="I132" s="0">
-        <x:v>16.12</x:v>
+        <x:v>17.13</x:v>
       </x:c>
       <x:c r="J132" s="0">
         <x:v>10.93</x:v>
       </x:c>
       <x:c r="K132" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="133" spans="1:11">
       <x:c r="A133" s="0" t="s">
-        <x:v>252</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="B133" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C133" s="0">
         <x:v>1590000</x:v>
@@ -5919,21 +5925,21 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="I133" s="0">
-        <x:v>36.5</x:v>
+        <x:v>37.02</x:v>
       </x:c>
       <x:c r="J133" s="0">
         <x:v>38.14</x:v>
       </x:c>
       <x:c r="K133" s="0" t="s">
-        <x:v>253</x:v>
+        <x:v>254</x:v>
       </x:c>
     </x:row>
     <x:row r="134" spans="1:11">
       <x:c r="A134" s="0" t="s">
-        <x:v>254</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="B134" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C134" s="0">
         <x:v>1989802</x:v>
@@ -5954,21 +5960,21 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I134" s="0">
-        <x:v>136</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="J134" s="0">
         <x:v>39.56</x:v>
       </x:c>
       <x:c r="K134" s="0" t="s">
-        <x:v>255</x:v>
+        <x:v>256</x:v>
       </x:c>
     </x:row>
     <x:row r="135" spans="1:11">
       <x:c r="A135" s="0" t="s">
-        <x:v>256</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B135" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C135" s="0" t="s">
         <x:v>13</x:v>
@@ -5989,7 +5995,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I135" s="0">
-        <x:v>541</x:v>
+        <x:v>549.5</x:v>
       </x:c>
       <x:c r="J135" s="0">
         <x:v>0</x:v>
@@ -5997,10 +6003,10 @@
     </x:row>
     <x:row r="136" spans="1:11">
       <x:c r="A136" s="0" t="s">
-        <x:v>257</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="B136" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C136" s="0">
         <x:v>300000</x:v>
@@ -6021,21 +6027,21 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I136" s="0">
-        <x:v>7.33</x:v>
+        <x:v>7.15</x:v>
       </x:c>
       <x:c r="J136" s="0">
         <x:v>4.56</x:v>
       </x:c>
       <x:c r="K136" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="137" spans="1:11">
       <x:c r="A137" s="0" t="s">
-        <x:v>258</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="B137" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C137" s="0">
         <x:v>76908759</x:v>
@@ -6056,21 +6062,21 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I137" s="0">
-        <x:v>34.62</x:v>
+        <x:v>38.08</x:v>
       </x:c>
       <x:c r="J137" s="0">
         <x:v>25.74</x:v>
       </x:c>
       <x:c r="K137" s="0" t="s">
-        <x:v>259</x:v>
+        <x:v>260</x:v>
       </x:c>
     </x:row>
     <x:row r="138" spans="1:11">
       <x:c r="A138" s="0" t="s">
-        <x:v>260</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="B138" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="C138" s="0">
         <x:v>8291656</x:v>
@@ -6091,21 +6097,21 @@
         <x:v>1.9</x:v>
       </x:c>
       <x:c r="I138" s="0">
-        <x:v>17.19</x:v>
+        <x:v>16.61</x:v>
       </x:c>
       <x:c r="J138" s="0">
         <x:v>15.2</x:v>
       </x:c>
       <x:c r="K138" s="0" t="s">
-        <x:v>185</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="139" spans="1:11">
       <x:c r="A139" s="0" t="s">
-        <x:v>261</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="B139" s="0" t="s">
-        <x:v>262</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="C139" s="0">
         <x:v>2975773</x:v>
@@ -6126,7 +6132,7 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="I139" s="0">
-        <x:v>24.66</x:v>
+        <x:v>24.28</x:v>
       </x:c>
       <x:c r="J139" s="0">
         <x:v>15.05</x:v>
@@ -6137,10 +6143,10 @@
     </x:row>
     <x:row r="140" spans="1:11">
       <x:c r="A140" s="0" t="s">
-        <x:v>263</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="B140" s="0" t="s">
-        <x:v>264</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="C140" s="0">
         <x:v>10994323</x:v>
@@ -6161,21 +6167,21 @@
         <x:v>5.09</x:v>
       </x:c>
       <x:c r="I140" s="0">
-        <x:v>12.72</x:v>
+        <x:v>13.59</x:v>
       </x:c>
       <x:c r="J140" s="0">
         <x:v>16.65</x:v>
       </x:c>
       <x:c r="K140" s="0" t="s">
-        <x:v>265</x:v>
+        <x:v>266</x:v>
       </x:c>
     </x:row>
     <x:row r="141" spans="1:11">
       <x:c r="A141" s="0" t="s">
-        <x:v>266</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="B141" s="0" t="s">
-        <x:v>267</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="C141" s="0">
         <x:v>36870641</x:v>
@@ -6196,21 +6202,21 @@
         <x:v>1.89</x:v>
       </x:c>
       <x:c r="I141" s="0">
-        <x:v>16.71</x:v>
+        <x:v>16.7</x:v>
       </x:c>
       <x:c r="J141" s="0">
         <x:v>11.29</x:v>
       </x:c>
       <x:c r="K141" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="142" spans="1:11">
       <x:c r="A142" s="0" t="s">
+        <x:v>269</x:v>
+      </x:c>
+      <x:c r="B142" s="0" t="s">
         <x:v>268</x:v>
-      </x:c>
-      <x:c r="B142" s="0" t="s">
-        <x:v>267</x:v>
       </x:c>
       <x:c r="C142" s="0">
         <x:v>5100000</x:v>
@@ -6231,21 +6237,21 @@
         <x:v>0.93</x:v>
       </x:c>
       <x:c r="I142" s="0">
-        <x:v>60</x:v>
+        <x:v>59.9</x:v>
       </x:c>
       <x:c r="J142" s="0">
         <x:v>30.45</x:v>
       </x:c>
       <x:c r="K142" s="0" t="s">
-        <x:v>269</x:v>
+        <x:v>270</x:v>
       </x:c>
     </x:row>
     <x:row r="143" spans="1:11">
       <x:c r="A143" s="0" t="s">
-        <x:v>270</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="B143" s="0" t="s">
-        <x:v>271</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="C143" s="0" t="s">
         <x:v>13</x:v>
@@ -6266,7 +6272,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I143" s="0">
-        <x:v>2.05</x:v>
+        <x:v>2.04</x:v>
       </x:c>
       <x:c r="J143" s="0">
         <x:v>0</x:v>
@@ -6277,7 +6283,7 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B144" s="0" t="s">
-        <x:v>272</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="C144" s="0">
         <x:v>5000000</x:v>
@@ -6298,21 +6304,21 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I144" s="0">
-        <x:v>9.93</x:v>
+        <x:v>10.2</x:v>
       </x:c>
       <x:c r="J144" s="0">
         <x:v>7.82</x:v>
       </x:c>
       <x:c r="K144" s="0" t="s">
-        <x:v>273</x:v>
+        <x:v>274</x:v>
       </x:c>
     </x:row>
     <x:row r="145" spans="1:11">
       <x:c r="A145" s="0" t="s">
-        <x:v>274</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="B145" s="0" t="s">
-        <x:v>275</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="C145" s="0">
         <x:v>905991</x:v>
@@ -6333,21 +6339,21 @@
         <x:v>0.13</x:v>
       </x:c>
       <x:c r="I145" s="0">
-        <x:v>17.46</x:v>
+        <x:v>16.67</x:v>
       </x:c>
       <x:c r="J145" s="0">
         <x:v>19.26</x:v>
       </x:c>
       <x:c r="K145" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="146" spans="1:11">
       <x:c r="A146" s="0" t="s">
-        <x:v>276</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="B146" s="0" t="s">
-        <x:v>277</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="C146" s="0" t="s">
         <x:v>13</x:v>
@@ -6368,7 +6374,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I146" s="0">
-        <x:v>41.22</x:v>
+        <x:v>40.82</x:v>
       </x:c>
       <x:c r="J146" s="0">
         <x:v>0</x:v>
@@ -6376,10 +6382,10 @@
     </x:row>
     <x:row r="147" spans="1:11">
       <x:c r="A147" s="0" t="s">
-        <x:v>256</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B147" s="0" t="s">
-        <x:v>278</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="C147" s="0" t="s">
         <x:v>13</x:v>
@@ -6400,7 +6406,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I147" s="0">
-        <x:v>541</x:v>
+        <x:v>549.5</x:v>
       </x:c>
       <x:c r="J147" s="0">
         <x:v>0</x:v>
@@ -6408,10 +6414,10 @@
     </x:row>
     <x:row r="148" spans="1:11">
       <x:c r="A148" s="0" t="s">
-        <x:v>279</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="B148" s="0" t="s">
-        <x:v>280</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="C148" s="0">
         <x:v>53584</x:v>
@@ -6432,7 +6438,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I148" s="0">
-        <x:v>257</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="J148" s="0">
         <x:v>154.36</x:v>
@@ -6443,10 +6449,10 @@
     </x:row>
     <x:row r="149" spans="1:11">
       <x:c r="A149" s="0" t="s">
-        <x:v>281</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="B149" s="0" t="s">
-        <x:v>282</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="C149" s="0">
         <x:v>7550000</x:v>
@@ -6467,21 +6473,21 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I149" s="0">
-        <x:v>14.51</x:v>
+        <x:v>14.2</x:v>
       </x:c>
       <x:c r="J149" s="0">
         <x:v>14.81</x:v>
       </x:c>
       <x:c r="K149" s="0" t="s">
-        <x:v>283</x:v>
+        <x:v>284</x:v>
       </x:c>
     </x:row>
     <x:row r="150" spans="1:11">
       <x:c r="A150" s="0" t="s">
-        <x:v>284</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="B150" s="0" t="s">
-        <x:v>285</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="C150" s="0">
         <x:v>2097716</x:v>
@@ -6502,21 +6508,21 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I150" s="0">
-        <x:v>1.23</x:v>
+        <x:v>1.22</x:v>
       </x:c>
       <x:c r="J150" s="0">
         <x:v>13.82</x:v>
       </x:c>
       <x:c r="K150" s="0" t="s">
-        <x:v>212</x:v>
+        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="151" spans="1:11">
       <x:c r="A151" s="0" t="s">
-        <x:v>286</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="B151" s="0" t="s">
-        <x:v>287</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="C151" s="0">
         <x:v>5185302</x:v>
@@ -6537,21 +6543,21 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I151" s="0">
-        <x:v>5.7</x:v>
+        <x:v>5.65</x:v>
       </x:c>
       <x:c r="J151" s="0">
         <x:v>7.15</x:v>
       </x:c>
       <x:c r="K151" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="152" spans="1:11">
       <x:c r="A152" s="0" t="s">
-        <x:v>288</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="B152" s="0" t="s">
-        <x:v>289</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C152" s="0">
         <x:v>669111</x:v>
@@ -6572,21 +6578,21 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I152" s="0">
-        <x:v>775</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="J152" s="0">
         <x:v>226</x:v>
       </x:c>
       <x:c r="K152" s="0" t="s">
-        <x:v>248</x:v>
+        <x:v>249</x:v>
       </x:c>
     </x:row>
     <x:row r="153" spans="1:11">
       <x:c r="A153" s="0" t="s">
-        <x:v>256</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B153" s="0" t="s">
-        <x:v>289</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="C153" s="0">
         <x:v>38840</x:v>
@@ -6607,21 +6613,21 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I153" s="0">
-        <x:v>541</x:v>
+        <x:v>549.5</x:v>
       </x:c>
       <x:c r="J153" s="0">
         <x:v>242.84</x:v>
       </x:c>
       <x:c r="K153" s="0" t="s">
-        <x:v>285</x:v>
+        <x:v>286</x:v>
       </x:c>
     </x:row>
     <x:row r="154" spans="1:11">
       <x:c r="A154" s="0" t="s">
-        <x:v>281</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="B154" s="0" t="s">
-        <x:v>290</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="C154" s="0">
         <x:v>2250000</x:v>
@@ -6642,21 +6648,21 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I154" s="0">
-        <x:v>14.51</x:v>
+        <x:v>14.2</x:v>
       </x:c>
       <x:c r="J154" s="0">
         <x:v>14.11</x:v>
       </x:c>
       <x:c r="K154" s="0" t="s">
-        <x:v>291</x:v>
+        <x:v>292</x:v>
       </x:c>
     </x:row>
     <x:row r="155" spans="1:11">
       <x:c r="A155" s="0" t="s">
-        <x:v>284</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="B155" s="0" t="s">
-        <x:v>292</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="C155" s="0">
         <x:v>1500000</x:v>
@@ -6677,21 +6683,21 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I155" s="0">
-        <x:v>1.23</x:v>
+        <x:v>1.22</x:v>
       </x:c>
       <x:c r="J155" s="0">
         <x:v>14.58</x:v>
       </x:c>
       <x:c r="K155" s="0" t="s">
-        <x:v>291</x:v>
+        <x:v>292</x:v>
       </x:c>
     </x:row>
     <x:row r="156" spans="1:11">
       <x:c r="A156" s="0" t="s">
-        <x:v>293</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="B156" s="0" t="s">
-        <x:v>294</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="C156" s="0">
         <x:v>1430040</x:v>
@@ -6712,7 +6718,7 @@
         <x:v>1.51</x:v>
       </x:c>
       <x:c r="I156" s="0">
-        <x:v>143.1</x:v>
+        <x:v>140.9</x:v>
       </x:c>
       <x:c r="J156" s="0">
         <x:v>138.67</x:v>
@@ -6723,10 +6729,10 @@
     </x:row>
     <x:row r="157" spans="1:11">
       <x:c r="A157" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B157" s="0" t="s">
-        <x:v>295</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="C157" s="0" t="s">
         <x:v>13</x:v>
@@ -6747,7 +6753,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I157" s="0">
-        <x:v>287.5</x:v>
+        <x:v>277.75</x:v>
       </x:c>
       <x:c r="J157" s="0">
         <x:v>0</x:v>
@@ -6755,10 +6761,10 @@
     </x:row>
     <x:row r="158" spans="1:11">
       <x:c r="A158" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B158" s="0" t="s">
-        <x:v>296</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="C158" s="0">
         <x:v>845945</x:v>
@@ -6779,21 +6785,21 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I158" s="0">
-        <x:v>3.89</x:v>
+        <x:v>3.78</x:v>
       </x:c>
       <x:c r="J158" s="0">
         <x:v>11.89</x:v>
       </x:c>
       <x:c r="K158" s="0" t="s">
-        <x:v>195</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="159" spans="1:11">
       <x:c r="A159" s="0" t="s">
-        <x:v>297</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="B159" s="0" t="s">
-        <x:v>298</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="C159" s="0">
         <x:v>21446</x:v>
@@ -6814,21 +6820,21 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I159" s="0">
-        <x:v>44.8</x:v>
+        <x:v>44.78</x:v>
       </x:c>
       <x:c r="J159" s="0">
         <x:v>94</x:v>
       </x:c>
       <x:c r="K159" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="160" spans="1:11">
       <x:c r="A160" s="0" t="s">
-        <x:v>299</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="B160" s="0" t="s">
-        <x:v>300</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="C160" s="0">
         <x:v>850000</x:v>
@@ -6849,21 +6855,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I160" s="0">
-        <x:v>6.99</x:v>
+        <x:v>6.94</x:v>
       </x:c>
       <x:c r="J160" s="0">
         <x:v>7.7</x:v>
       </x:c>
       <x:c r="K160" s="0" t="s">
-        <x:v>230</x:v>
+        <x:v>231</x:v>
       </x:c>
     </x:row>
     <x:row r="161" spans="1:11">
       <x:c r="A161" s="0" t="s">
-        <x:v>301</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="B161" s="0" t="s">
-        <x:v>302</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="C161" s="0">
         <x:v>15000000</x:v>
@@ -6884,21 +6890,21 @@
         <x:v>0.22</x:v>
       </x:c>
       <x:c r="I161" s="0">
-        <x:v>3.1</x:v>
+        <x:v>3.12</x:v>
       </x:c>
       <x:c r="J161" s="0">
         <x:v>1.6</x:v>
       </x:c>
       <x:c r="K161" s="0" t="s">
-        <x:v>303</x:v>
+        <x:v>304</x:v>
       </x:c>
     </x:row>
     <x:row r="162" spans="1:11">
       <x:c r="A162" s="0" t="s">
-        <x:v>304</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="B162" s="0" t="s">
-        <x:v>305</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="C162" s="0">
         <x:v>6397124</x:v>
@@ -6919,13 +6925,13 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I162" s="0">
-        <x:v>4.07</x:v>
+        <x:v>4.06</x:v>
       </x:c>
       <x:c r="J162" s="0">
         <x:v>19.21</x:v>
       </x:c>
       <x:c r="K162" s="0" t="s">
-        <x:v>306</x:v>
+        <x:v>307</x:v>
       </x:c>
     </x:row>
     <x:row r="163" spans="1:11">
@@ -6933,7 +6939,7 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="B163" s="0" t="s">
-        <x:v>307</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="C163" s="0">
         <x:v>17495257</x:v>
@@ -6954,21 +6960,21 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I163" s="0">
-        <x:v>17.87</x:v>
+        <x:v>17.9</x:v>
       </x:c>
       <x:c r="J163" s="0">
         <x:v>23.4</x:v>
       </x:c>
       <x:c r="K163" s="0" t="s">
-        <x:v>308</x:v>
+        <x:v>309</x:v>
       </x:c>
     </x:row>
     <x:row r="164" spans="1:11">
       <x:c r="A164" s="0" t="s">
-        <x:v>309</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="B164" s="0" t="s">
-        <x:v>310</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="C164" s="0">
         <x:v>9350000</x:v>
@@ -6989,13 +6995,13 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="I164" s="0">
-        <x:v>2.45</x:v>
+        <x:v>2.3</x:v>
       </x:c>
       <x:c r="J164" s="0">
         <x:v>7.44</x:v>
       </x:c>
       <x:c r="K164" s="0" t="s">
-        <x:v>311</x:v>
+        <x:v>312</x:v>
       </x:c>
     </x:row>
     <x:row r="165" spans="1:11">
@@ -7003,7 +7009,7 @@
         <x:v>146</x:v>
       </x:c>
       <x:c r="B165" s="0" t="s">
-        <x:v>312</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="C165" s="0">
         <x:v>1468255</x:v>
@@ -7024,21 +7030,21 @@
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="I165" s="0">
-        <x:v>23.38</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J165" s="0">
         <x:v>51.7</x:v>
       </x:c>
       <x:c r="K165" s="0" t="s">
-        <x:v>313</x:v>
+        <x:v>314</x:v>
       </x:c>
     </x:row>
     <x:row r="166" spans="1:11">
       <x:c r="A166" s="0" t="s">
-        <x:v>314</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="B166" s="0" t="s">
-        <x:v>315</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="C166" s="0">
         <x:v>500000</x:v>
@@ -7059,21 +7065,21 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I166" s="0">
-        <x:v>2.24</x:v>
+        <x:v>2.31</x:v>
       </x:c>
       <x:c r="J166" s="0">
         <x:v>26.8</x:v>
       </x:c>
       <x:c r="K166" s="0" t="s">
-        <x:v>189</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="167" spans="1:11">
       <x:c r="A167" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B167" s="0" t="s">
-        <x:v>316</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="C167" s="0">
         <x:v>725000</x:v>
@@ -7094,21 +7100,21 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="I167" s="0">
-        <x:v>39.3</x:v>
+        <x:v>38.94</x:v>
       </x:c>
       <x:c r="J167" s="0">
         <x:v>66.95</x:v>
       </x:c>
       <x:c r="K167" s="0" t="s">
-        <x:v>317</x:v>
+        <x:v>318</x:v>
       </x:c>
     </x:row>
     <x:row r="168" spans="1:11">
       <x:c r="A168" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="B168" s="0" t="s">
-        <x:v>318</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="C168" s="0">
         <x:v>1060056</x:v>
@@ -7129,21 +7135,21 @@
         <x:v>0.44</x:v>
       </x:c>
       <x:c r="I168" s="0">
-        <x:v>225</x:v>
+        <x:v>223.8</x:v>
       </x:c>
       <x:c r="J168" s="0">
         <x:v>57.32</x:v>
       </x:c>
       <x:c r="K168" s="0" t="s">
-        <x:v>319</x:v>
+        <x:v>320</x:v>
       </x:c>
     </x:row>
     <x:row r="169" spans="1:11">
       <x:c r="A169" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B169" s="0" t="s">
-        <x:v>320</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="C169" s="0">
         <x:v>132750000</x:v>
@@ -7164,21 +7170,21 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I169" s="0">
-        <x:v>2.77</x:v>
+        <x:v>2.82</x:v>
       </x:c>
       <x:c r="J169" s="0">
         <x:v>4.26</x:v>
       </x:c>
       <x:c r="K169" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="170" spans="1:11">
       <x:c r="A170" s="0" t="s">
-        <x:v>321</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="B170" s="0" t="s">
-        <x:v>322</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="C170" s="0">
         <x:v>373000</x:v>
@@ -7199,21 +7205,21 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I170" s="0">
-        <x:v>8.46</x:v>
+        <x:v>8.35</x:v>
       </x:c>
       <x:c r="J170" s="0">
         <x:v>63.77</x:v>
       </x:c>
       <x:c r="K170" s="0" t="s">
-        <x:v>323</x:v>
+        <x:v>324</x:v>
       </x:c>
     </x:row>
     <x:row r="171" spans="1:11">
       <x:c r="A171" s="0" t="s">
-        <x:v>324</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="B171" s="0" t="s">
-        <x:v>325</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="C171" s="0">
         <x:v>10000000</x:v>
@@ -7234,21 +7240,21 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I171" s="0">
-        <x:v>10.6</x:v>
+        <x:v>10.46</x:v>
       </x:c>
       <x:c r="J171" s="0">
         <x:v>13.33</x:v>
       </x:c>
       <x:c r="K171" s="0" t="s">
-        <x:v>326</x:v>
+        <x:v>327</x:v>
       </x:c>
     </x:row>
     <x:row r="172" spans="1:11">
       <x:c r="A172" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B172" s="0" t="s">
-        <x:v>327</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="C172" s="0">
         <x:v>66142950</x:v>
@@ -7269,21 +7275,21 @@
         <x:v>2.71</x:v>
       </x:c>
       <x:c r="I172" s="0">
-        <x:v>7.12</x:v>
+        <x:v>7.06</x:v>
       </x:c>
       <x:c r="J172" s="0">
         <x:v>5.82</x:v>
       </x:c>
       <x:c r="K172" s="0" t="s">
-        <x:v>328</x:v>
+        <x:v>329</x:v>
       </x:c>
     </x:row>
     <x:row r="173" spans="1:11">
       <x:c r="A173" s="0" t="s">
-        <x:v>329</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="B173" s="0" t="s">
-        <x:v>330</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="C173" s="0">
         <x:v>3081843</x:v>
@@ -7304,13 +7310,13 @@
         <x:v>0.66</x:v>
       </x:c>
       <x:c r="I173" s="0">
-        <x:v>5.68</x:v>
+        <x:v>5.67</x:v>
       </x:c>
       <x:c r="J173" s="0">
         <x:v>14.27</x:v>
       </x:c>
       <x:c r="K173" s="0" t="s">
-        <x:v>272</x:v>
+        <x:v>273</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>